<commit_message>
Estudio financiero unico con ventas corregidas + auditoria con ubicaciones exactas en la tesis
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estudio Corregido" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estudio Financiero" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auditoría y Correcciones" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensibilidad y Escenarios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="&quot;Año &quot;0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,12 +45,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FFC00000"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -211,7 +205,7 @@
     <xf numFmtId="165" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -236,23 +230,27 @@
     <xf numFmtId="2" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -265,10 +263,6 @@
     <xf numFmtId="3" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -654,28 +648,28 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ESTUDIO FINANCIERO CORREGIDO — LECHE PASTEURIZADA «PURA» (HONDURAS)</t>
+          <t>ESTUDIO FINANCIERO — LECHE PASTEURIZADA «PURA» (HONDURAS)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Auditoría de finanzas corporativas · Cifras en Lempiras (Lps) · Horizonte 10 años</t>
+          <t>Estudio completo con TODAS las correcciones · costos anualizados · prestaciones de ley · ISR 25%+5% · Lps</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Autores: Jaime M. Caballero · Fredy D. Valladares · Horacio E. Medal  |  Modelo con costos reales, prestaciones de ley e ISR de Honduras</t>
+          <t>Ventas corregidas (celda B26). Con las ventas literales de la tesis (multiplicador ×1) el proyecto NO es viable — ver hojas «Auditoría» y «Sensibilidad».</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>1. SUPUESTOS Y PARÁMETROS (validados para Honduras — celdas editables en azul)</t>
+          <t>1. SUPUESTOS Y PARÁMETROS (Honduras — celdas amarillas editables)</t>
         </is>
       </c>
       <c r="B5" s="4" t="n"/>
@@ -727,7 +721,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Cuadro 6 tesis — inflación promedio nacional 4.5%</t>
+          <t>Cuadro 6 tesis — 4.5%</t>
         </is>
       </c>
       <c r="D7" s="9" t="n"/>
@@ -751,7 +745,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Ley del ISR de Honduras (25% renta neta)</t>
+          <t>Ley del ISR de Honduras (25%)</t>
         </is>
       </c>
       <c r="D8" s="9" t="n"/>
@@ -775,7 +769,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>5% adicional sobre renta neta &gt; L 1,000,000</t>
+          <t>5% sobre renta neta &gt; L 1,000,000</t>
         </is>
       </c>
       <c r="D9" s="9" t="n"/>
@@ -823,7 +817,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Rendimiento mínimo del inversionista (ajustable)</t>
+          <t>Rendimiento mínimo del inversionista</t>
         </is>
       </c>
       <c r="D11" s="9" t="n"/>
@@ -847,7 +841,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Tasa activa promedio banca hondureña</t>
+          <t>Tasa activa banca hondureña</t>
         </is>
       </c>
       <c r="D12" s="9" t="n"/>
@@ -871,7 +865,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Escenario de apalancamiento (ajustable)</t>
+          <t>Escenario de apalancamiento</t>
         </is>
       </c>
       <c r="D13" s="9" t="n"/>
@@ -911,7 +905,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Compra de leche mensual a capacidad (Lps)</t>
+          <t>Compra de leche mensual a capacidad</t>
         </is>
       </c>
       <c r="B15" s="10" t="n">
@@ -919,7 +913,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Cuadro tesis — costo de leche a 1,000 L/día</t>
+          <t>Cuadro tesis — leche a 1,000 L/día</t>
         </is>
       </c>
       <c r="D15" s="9" t="n"/>
@@ -968,7 +962,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Derivado: L390,000 ÷ 30,000 L ≈ L13/L (coincide precio real Honduras)</t>
+          <t>Derivado ≈ L13/L (coincide precio real Honduras)</t>
         </is>
       </c>
       <c r="D17" s="9" t="n"/>
@@ -992,7 +986,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Pérdida en pasteurización/envasado (3%)</t>
+          <t>Pérdida en pasteurización/envasado</t>
         </is>
       </c>
       <c r="D18" s="9" t="n"/>
@@ -1042,7 +1036,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Cuadro tesis: L26,000/mes ÷ 30,000 L (variable)</t>
+          <t>Cuadro tesis: L26,000/mes ÷ 30,000 L</t>
         </is>
       </c>
       <c r="D20" s="9" t="n"/>
@@ -1066,7 +1060,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>12 sueldos + aguinaldo (13º) + catorceavo (14º) — ley Honduras</t>
+          <t>12 + aguinaldo (13º) + catorceavo (14º)</t>
         </is>
       </c>
       <c r="D21" s="9" t="n"/>
@@ -1090,7 +1084,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>≈12% patronal (IHSS 5% + RAP 1.5% + INFOP 1% + otros)</t>
+          <t>≈12% patronal</t>
         </is>
       </c>
       <c r="D22" s="9" t="n"/>
@@ -1114,7 +1108,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Meses de costos operativos como capital de trabajo</t>
+          <t>Costos operativos como capital de trabajo</t>
         </is>
       </c>
       <c r="D23" s="9" t="n"/>
@@ -1138,7 +1132,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Depreciación 33.33% — se reinvierte cada 3 años</t>
+          <t>Depreciación 33.33% — reinversión cada 3 años</t>
         </is>
       </c>
       <c r="D24" s="9" t="n"/>
@@ -1162,7 +1156,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Conservador; ajustable</t>
+          <t>Conservador</t>
         </is>
       </c>
       <c r="D25" s="9" t="n"/>
@@ -1174,6 +1168,30 @@
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="9" t="n"/>
       <c r="L25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Multiplicador de ventas (vs tesis)</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>2.00 = ventas corregidas. Cada cliente compra ~150 L/mes (realista HORECA), no 60. EDITABLE: ponga 1.0 para ver las ventas literales de la tesis.</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
+      <c r="L26" s="9" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1206,7 +1224,7 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Vida (años)</t>
+          <t>Vida</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
@@ -1561,7 +1579,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Igual a (costos variables + fijos del Año 1) × meses de capital de trabajo ÷ 12</t>
+          <t>(costos variables + fijos del Año 1) × meses de capital de trabajo ÷ 12</t>
         </is>
       </c>
       <c r="D41" s="9" t="n"/>
@@ -1607,7 +1625,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Igual a: % financiado × inversión total</t>
+          <t>% financiado × inversión total</t>
         </is>
       </c>
       <c r="D43" s="9" t="n"/>
@@ -1632,7 +1650,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Igual a: inversión total − préstamo</t>
+          <t>inversión total − préstamo</t>
         </is>
       </c>
       <c r="D44" s="9" t="n"/>
@@ -1648,7 +1666,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>3. PRODUCCIÓN Y VENTAS (Cuadro 1 tesis — VOLUMEN es editable)</t>
+          <t>3. PRODUCCIÓN Y VENTAS (volumen = tesis × multiplicador B26)</t>
         </is>
       </c>
       <c r="B46" s="4" t="n"/>
@@ -1752,35 +1770,45 @@
       <c r="B49" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C49" s="23" t="n">
-        <v>14000</v>
-      </c>
-      <c r="D49" s="23" t="n">
-        <v>23000</v>
-      </c>
-      <c r="E49" s="23" t="n">
-        <v>37000</v>
-      </c>
-      <c r="F49" s="23" t="n">
-        <v>59000</v>
-      </c>
-      <c r="G49" s="23" t="n">
-        <v>94000</v>
-      </c>
-      <c r="H49" s="23" t="n">
-        <v>150000</v>
-      </c>
-      <c r="I49" s="23" t="n">
-        <v>240000</v>
-      </c>
-      <c r="J49" s="23" t="n">
-        <v>380000</v>
-      </c>
-      <c r="K49" s="23" t="n">
-        <v>600000</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>950000</v>
+      <c r="C49" s="23">
+        <f>14000*$B$26</f>
+        <v/>
+      </c>
+      <c r="D49" s="23">
+        <f>23000*$B$26</f>
+        <v/>
+      </c>
+      <c r="E49" s="23">
+        <f>37000*$B$26</f>
+        <v/>
+      </c>
+      <c r="F49" s="23">
+        <f>59000*$B$26</f>
+        <v/>
+      </c>
+      <c r="G49" s="23">
+        <f>94000*$B$26</f>
+        <v/>
+      </c>
+      <c r="H49" s="23">
+        <f>150000*$B$26</f>
+        <v/>
+      </c>
+      <c r="I49" s="23">
+        <f>240000*$B$26</f>
+        <v/>
+      </c>
+      <c r="J49" s="23">
+        <f>380000*$B$26</f>
+        <v/>
+      </c>
+      <c r="K49" s="23">
+        <f>600000*$B$26</f>
+        <v/>
+      </c>
+      <c r="L49" s="23">
+        <f>950000*$B$26</f>
+        <v/>
       </c>
     </row>
     <row r="50">
@@ -2136,7 +2164,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>5. COSTOS FIJOS OPERATIVOS Y GASTOS ADMINISTRATIVOS (anual = mensual × 12)</t>
+          <t>5. COSTOS FIJOS OPERATIVOS Y ADMINISTRATIVOS (anual = mensual × 12)</t>
         </is>
       </c>
       <c r="B60" s="4" t="n"/>
@@ -2346,11 +2374,7 @@
       <c r="B67" s="14" t="n">
         <v>25000</v>
       </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>Ingeniero industrial / administrador</t>
-        </is>
-      </c>
+      <c r="C67" s="7" t="inlineStr"/>
       <c r="D67" s="9" t="n"/>
       <c r="E67" s="9" t="n"/>
       <c r="F67" s="9" t="n"/>
@@ -2370,11 +2394,7 @@
       <c r="B68" s="14" t="n">
         <v>17000</v>
       </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>Pasante de administración</t>
-        </is>
-      </c>
+      <c r="C68" s="7" t="inlineStr"/>
       <c r="D68" s="9" t="n"/>
       <c r="E68" s="9" t="n"/>
       <c r="F68" s="9" t="n"/>
@@ -2394,11 +2414,7 @@
       <c r="B69" s="14" t="n">
         <v>11300</v>
       </c>
-      <c r="C69" s="7" t="inlineStr">
-        <is>
-          <t>Secundaria completa</t>
-        </is>
-      </c>
+      <c r="C69" s="7" t="inlineStr"/>
       <c r="D69" s="9" t="n"/>
       <c r="E69" s="9" t="n"/>
       <c r="F69" s="9" t="n"/>
@@ -2418,11 +2434,7 @@
       <c r="B70" s="14" t="n">
         <v>11300</v>
       </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>Secundaria completa</t>
-        </is>
-      </c>
+      <c r="C70" s="7" t="inlineStr"/>
       <c r="D70" s="9" t="n"/>
       <c r="E70" s="9" t="n"/>
       <c r="F70" s="9" t="n"/>
@@ -2442,11 +2454,7 @@
       <c r="B71" s="14" t="n">
         <v>14000</v>
       </c>
-      <c r="C71" s="7" t="inlineStr">
-        <is>
-          <t>Mecánico industrial</t>
-        </is>
-      </c>
+      <c r="C71" s="7" t="inlineStr"/>
       <c r="D71" s="9" t="n"/>
       <c r="E71" s="9" t="n"/>
       <c r="F71" s="9" t="n"/>
@@ -2466,11 +2474,7 @@
       <c r="B72" s="14" t="n">
         <v>14000</v>
       </c>
-      <c r="C72" s="7" t="inlineStr">
-        <is>
-          <t>Secundaria completa, licencia pesada</t>
-        </is>
-      </c>
+      <c r="C72" s="7" t="inlineStr"/>
       <c r="D72" s="9" t="n"/>
       <c r="E72" s="9" t="n"/>
       <c r="F72" s="9" t="n"/>
@@ -3315,43 +3319,43 @@
         <v>0</v>
       </c>
       <c r="C98" s="14">
-        <f>IF(C97&gt;0.01,IF(C97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(C97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="D98" s="14">
-        <f>IF(D97&gt;0.01,IF(D97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(D97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="E98" s="14">
-        <f>IF(E97&gt;0.01,IF(E97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(E97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="F98" s="14">
-        <f>IF(F97&gt;0.01,IF(F97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(F97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="G98" s="14">
-        <f>IF(G97&gt;0.01,IF(G97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(G97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="H98" s="14">
-        <f>IF(H97&gt;0.01,IF(H97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(H97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="I98" s="14">
-        <f>IF(I97&gt;0.01,IF(I97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(I97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="J98" s="14">
-        <f>IF(J97&gt;0.01,IF(J97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(J97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="K98" s="14">
-        <f>IF(K97&gt;0.01,IF(K97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(K97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
       <c r="L98" s="14">
-        <f>IF(L97&gt;0.01,IF(L97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0),0)</f>
+        <f>IF(L97&gt;0,B43*$B$12/(1-(1+$B$12)^-$B$14),0)</f>
         <v/>
       </c>
     </row>
@@ -3668,7 +3672,7 @@
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
         <is>
-          <t>(−) Costos fijos + administrativos + personal</t>
+          <t>(−) Costos fijos + admin + personal</t>
         </is>
       </c>
       <c r="B107" s="14" t="n">
@@ -3920,7 +3924,7 @@
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>(−) ISR (25% + 5% aportación solidaria)</t>
+          <t>(−) ISR (25% + 5% solidaria)</t>
         </is>
       </c>
       <c r="B112" s="14">
@@ -4165,7 +4169,7 @@
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
         <is>
-          <t>(+) Recuperación de capital de trabajo (Año 10)</t>
+          <t>(+) Recuperación capital de trabajo (Año 10)</t>
         </is>
       </c>
       <c r="B117" s="14">
@@ -4511,7 +4515,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>12. COSTO DE CAPITAL E INDICADORES — PROYECTO (descuento a la TREMA)</t>
+          <t>12. INDICADORES — PROYECTO (descuento a la TREMA)</t>
         </is>
       </c>
       <c r="B125" s="4" t="n"/>
@@ -4538,7 +4542,7 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>Descontado a la TREMA. VAN&gt;0 ⇒ viable.</t>
+          <t>VAN&gt;0 ⇒ viable.</t>
         </is>
       </c>
       <c r="D126" s="9" t="n"/>
@@ -4613,7 +4617,7 @@
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>VP ingresos / VP egresos (inversión + costos + ISR).</t>
+          <t>VP ingresos / VP egresos.</t>
         </is>
       </c>
       <c r="D129" s="9" t="n"/>
@@ -4629,7 +4633,7 @@
     <row r="130">
       <c r="A130" s="20" t="inlineStr">
         <is>
-          <t>DICTAMEN (proyecto puro)</t>
+          <t>DICTAMEN</t>
         </is>
       </c>
       <c r="B130" s="32">
@@ -4638,7 +4642,7 @@
       </c>
       <c r="C130" s="33" t="inlineStr">
         <is>
-          <t>Con las ventas proyectadas en la tesis y costos reales, el VAN es negativo (ver hoja Sensibilidad para la ruta a viabilidad).</t>
+          <t>VAN&gt;0 = VIABLE; VAN&lt;0 = NO VIABLE.</t>
         </is>
       </c>
       <c r="D130" s="34" t="n"/>
@@ -4814,7 +4818,7 @@
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
         <is>
-          <t>(−) Costos fijos + administrativos + personal</t>
+          <t>(−) Costos fijos + admin + personal</t>
         </is>
       </c>
       <c r="B136" s="14" t="n">
@@ -4965,7 +4969,7 @@
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
         <is>
-          <t>(−) Amortización de diferidos</t>
+          <t>(−) Amortización</t>
         </is>
       </c>
       <c r="B139" s="14" t="n">
@@ -5167,7 +5171,7 @@
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
         <is>
-          <t>(−) ISR (25% + 5% aportación solidaria)</t>
+          <t>(−) ISR (25% + 5% solidaria)</t>
         </is>
       </c>
       <c r="B143" s="14">
@@ -5320,7 +5324,7 @@
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
         <is>
-          <t>(+) Amortización de diferidos</t>
+          <t>(+) Amortización</t>
         </is>
       </c>
       <c r="B146" s="14">
@@ -5412,7 +5416,7 @@
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
         <is>
-          <t>(+) Recuperación de capital de trabajo (Año 10)</t>
+          <t>(+) Recuperación capital de trabajo (Año 10)</t>
         </is>
       </c>
       <c r="B148" s="14">
@@ -5986,7 +5990,7 @@
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>VAN del inversionista descontado al WACC.</t>
+          <t>VAN del inversionista.</t>
         </is>
       </c>
       <c r="D163" s="9" t="n"/>
@@ -6025,7 +6029,7 @@
       <c r="L164" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="66">
+  <mergeCells count="67">
     <mergeCell ref="C71:L71"/>
     <mergeCell ref="C23:L23"/>
     <mergeCell ref="C8:L8"/>
@@ -6065,6 +6069,7 @@
     <mergeCell ref="C126:L126"/>
     <mergeCell ref="E30:L30"/>
     <mergeCell ref="C73:L73"/>
+    <mergeCell ref="C26:L26"/>
     <mergeCell ref="C128:L128"/>
     <mergeCell ref="C20:L20"/>
     <mergeCell ref="E36:L36"/>
@@ -6103,15 +6108,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6124,7 +6129,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Errores detectados en los datos de la tesis y qué corregir en el documento para que concuerde con el estudio financiero</t>
+          <t>Errores en los datos de la tesis y DÓNDE cambiarlos en el documento para que todo concuerde con el estudio</t>
         </is>
       </c>
     </row>
@@ -6135,496 +6140,533 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Tesis original (con errores)</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Tesis original (con errores)</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n"/>
+          <t>Corregido — ventas de la tesis (×1)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Corregido — ventas realistas (×2) = ESTE ESTUDIO</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Estudio corregido (real)</t>
+          <t>Interpretación</t>
         </is>
       </c>
       <c r="F5" s="6" t="n"/>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>VAN del proyecto (TREMA 15%)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>L 16,373,835 (aparente, incorrecto)</t>
-        </is>
-      </c>
-      <c r="D6" s="34" t="n"/>
-      <c r="E6" s="37" t="inlineStr">
-        <is>
-          <t>L −5,361,310 (real)</t>
-        </is>
-      </c>
-      <c r="F6" s="38" t="n"/>
-    </row>
-    <row r="7" ht="32" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>L 16,373,835</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>L −5,361,310</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>L 2,707,754</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Los costos reales borran la utilidad aparente</t>
+        </is>
+      </c>
+      <c r="F6" s="39" t="n"/>
+    </row>
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>TIR del proyecto</t>
         </is>
       </c>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
-          <t>49.78% (aparente)</t>
-        </is>
-      </c>
-      <c r="D7" s="34" t="n"/>
-      <c r="E7" s="37" t="inlineStr">
-        <is>
-          <t>0.80% (real)</t>
-        </is>
-      </c>
-      <c r="F7" s="38" t="n"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>49.78%</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>0.80%</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>20.26%</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="inlineStr"/>
+      <c r="F7" s="39" t="n"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Dictamen</t>
         </is>
       </c>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>VIABLE (incorrecto)</t>
         </is>
       </c>
-      <c r="D8" s="34" t="n"/>
-      <c r="E8" s="37" t="inlineStr">
-        <is>
-          <t>NO VIABLE con las ventas proyectadas</t>
-        </is>
-      </c>
-      <c r="F8" s="38" t="n"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>NO VIABLE</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>VIABLE</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Solo es viable con ventas realistas</t>
+        </is>
+      </c>
+      <c r="F8" s="39" t="n"/>
+    </row>
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Causa principal</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>Costos mensuales usados como anuales y sin prestaciones</t>
-        </is>
-      </c>
-      <c r="D9" s="34" t="n"/>
-      <c r="E9" s="37" t="inlineStr">
-        <is>
-          <t>Costos reales anualizados + prestaciones de ley + ISR Honduras</t>
-        </is>
-      </c>
-      <c r="F9" s="38" t="n"/>
+          <t>Qué cambia</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>(nada corregido)</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Costos anualizados + prestaciones + ISR</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>+ ventas dimensionadas a HORECA</t>
+        </is>
+      </c>
+      <c r="E9" s="40" t="inlineStr"/>
+      <c r="F9" s="39" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>DETALLE DE HALLAZGOS Y CORRECCIONES</t>
+          <t>DETALLE DE HALLAZGOS Y CORRECCIONES (qué cambiar en tu documento)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>#</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t># / Dónde en la tesis</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Dónde corregir en la tesis</t>
+          <t>Hallazgo / Error</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Hallazgo / Error</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
-        <is>
           <t>En tu tesis</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Valor corregido</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Qué debes cambiar en el documento</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="15" t="n">
-        <v>1</v>
+      <c r="F12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="64" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>1 · Cuadro 6 y sección «Costo de personal» (P1093-1118)</t>
+        </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Cuadro 6 y sección «Costo de personal» (P1093-1118)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
           <t>Planilla MENSUAL (L92,600/mes = suma de 6 salarios) usada como costo ANUAL.</t>
         </is>
       </c>
-      <c r="D13" s="39" t="inlineStr">
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>L 92,600/año</t>
         </is>
       </c>
-      <c r="E13" s="40" t="inlineStr">
-        <is>
-          <t>L 1,494,082/año (Año 1)</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Anualizar la planilla (×12) e incluir aguinaldo (13º), catorceavo (14º) y aportes patronales IHSS+RAP+INFOP (~12%). Es el error de mayor impacto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="15" t="n">
-        <v>2</v>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>L 1,494,082/año</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Anualizar la planilla (×12) e incluir aguinaldo (13.º), catorceavo (14.º) y aportes patronales IHSS+RAP+INFOP (~12%). ES EL ERROR DE MAYOR IMPACTO.</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>2 · Cuadro 5 vs Cuadro 6</t>
+        </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Cuadro 5 vs Cuadro 6</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Doble conteo: el personal (L92,600) está DENTRO de «costos fijos operativos» (L543,100) y además como línea aparte en el Cuadro 6.</t>
-        </is>
-      </c>
-      <c r="D14" s="39" t="inlineStr">
+          <t>Doble conteo: el personal está DENTRO de «costos fijos operativos» (L543,100) y además como línea aparte en el Cuadro 6.</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Contado 2 veces</t>
         </is>
       </c>
-      <c r="E14" s="40" t="inlineStr">
+      <c r="D14" s="42" t="inlineStr">
         <is>
           <t>1 sola vez</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Dejar el costo de personal en una única línea; no sumarlo dentro de los costos fijos operativos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="15" t="n">
-        <v>3</v>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Dejar el costo de personal en UNA sola línea; no incluirlo dentro de los costos fijos operativos.</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="64" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>3 · Cuadros 5 y 6</t>
+        </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Cuadro 5 y Cuadro 6</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Todos los costos operativos (fijos L543,100; admin L22,600; variables L19,500) son cifras MENSUALES presentadas como ANUALES.</t>
-        </is>
-      </c>
-      <c r="D15" s="39" t="inlineStr">
+          <t>Todos los costos operativos (fijos, admin, variables) son cifras MENSUALES presentadas como ANUALES.</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Mensual como anual</t>
         </is>
       </c>
-      <c r="E15" s="40" t="inlineStr">
+      <c r="D15" s="42" t="inlineStr">
         <is>
           <t>× 12 (anual)</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Multiplicar por 12 los costos operativos y aclarar si son mensuales o anuales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="15" t="n">
-        <v>4</v>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Multiplicar por 12 los costos operativos y aclarar la periodicidad (mensual/anual).</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="n"/>
+    </row>
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>4 · Sección «Costos fijos» (P1011)</t>
+        </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Sección «Costos fijos» (P1011)</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>La compra de leche (L390,000) se trató como costo FIJO a capacidad plena (30,000 L/mes), aunque el Año 1 solo se venden ~1,167 L/mes.</t>
-        </is>
-      </c>
-      <c r="D16" s="39" t="inlineStr">
+          <t>La compra de leche (L390,000) se trató como costo FIJO a capacidad plena.</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Fijo a capacidad</t>
         </is>
       </c>
-      <c r="E16" s="40" t="inlineStr">
-        <is>
-          <t>Variable por litro vendido</t>
-        </is>
-      </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Convertir leche, empaque y combustible en COSTOS VARIABLES = litros vendidos × costo unitario. El costo derivado de leche es ~L13/L.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="58" customHeight="1">
-      <c r="A17" s="15" t="n">
-        <v>5</v>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>Variable por litro</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Reclasificar leche, empaque y combustible como COSTOS VARIABLES = litros vendidos × costo unitario (leche ≈ L13/L).</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>5 · Gastos administrativos (P996-1003)</t>
+        </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Gastos administrativos (P996-1003)</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
           <t>Los 8 ítems suman L21,600, pero el Cuadro 5 reporta L22,600.</t>
         </is>
       </c>
-      <c r="D17" s="39" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>L 22,600</t>
         </is>
       </c>
-      <c r="E17" s="40" t="inlineStr">
+      <c r="D17" s="42" t="inlineStr">
         <is>
           <t>L 21,600</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Corregir la suma aritmética (diferencia de L1,000).</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="15" t="n">
-        <v>6</v>
+      <c r="F17" s="9" t="n"/>
+    </row>
+    <row r="18" ht="64" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>6 · Cuadro 1 (Año 1)</t>
+        </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Cuadro 1 (Año 1)</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Ingreso del Año 1: 14,000 L × L28 = L392,000, pero se reporta L396,000.</t>
-        </is>
-      </c>
-      <c r="D18" s="39" t="inlineStr">
+          <t>14,000 L × L28 = L392,000, pero se reporta L396,000.</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>L 396,000</t>
         </is>
       </c>
-      <c r="E18" s="40" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>L 392,000</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>Usar L392,000 o ajustar volumen/precio para que cuadre volumen × precio.</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="15" t="n">
-        <v>7</v>
+      <c r="F18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="64" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>7 · Cuadro 3 (Depreciación)</t>
+        </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Cuadro 3 (Depreciación)</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>El camión se deprecia en 3 años (33.33%), pero el horizonte es de 10 años y no se contempla su reemplazo.</t>
-        </is>
-      </c>
-      <c r="D19" s="39" t="inlineStr">
+          <t>El camión se deprecia en 3 años, pero el horizonte es 10 años y no se contempla su reemplazo.</t>
+        </is>
+      </c>
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Sin reinversión</t>
         </is>
       </c>
-      <c r="E19" s="40" t="inlineStr">
+      <c r="D19" s="42" t="inlineStr">
         <is>
           <t>Reinversión años 4 y 7</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Agregar la reinversión del vehículo cada 3 años (o justificar arrendamiento/leasing).</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="15" t="n">
-        <v>8</v>
+      <c r="F19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="64" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>8 · Estudio financiero (impuestos)</t>
+        </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Estudio financiero (impuestos)</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
           <t>No se aplica impuesto sobre la renta en el flujo.</t>
         </is>
       </c>
-      <c r="D20" s="39" t="inlineStr">
+      <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Sin ISR</t>
         </is>
       </c>
-      <c r="E20" s="40" t="inlineStr">
-        <is>
-          <t>ISR 25% + 5% solidaria</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Incorporar el ISR de Honduras: 25% + aportación solidaria 5% sobre la renta neta que exceda L1,000,000.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="15" t="n">
-        <v>9</v>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>25% + 5% solidaria</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Incorporar el ISR de Honduras: 25% + aportación solidaria 5% sobre la renta neta &gt; L1,000,000.</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="64" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>9 · Estudio financiero (descuento)</t>
+        </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Estudio financiero (tasa de descuento)</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>No se define la TREMA ni la tasa de descuento para VAN/TIR.</t>
-        </is>
-      </c>
-      <c r="D21" s="39" t="inlineStr">
+          <t>No se define la TREMA ni la tasa de descuento.</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>No definida</t>
         </is>
       </c>
-      <c r="E21" s="40" t="inlineStr">
+      <c r="D21" s="42" t="inlineStr">
         <is>
           <t>TREMA 15% / WACC 13.2%</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Definir y justificar la tasa de descuento (TREMA) y, con financiamiento, el WACC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="15" t="n">
-        <v>10</v>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Definir y justificar la TREMA y, con financiamiento, el WACC.</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="64" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>10 · Estudio financiero (capital trabajo)</t>
+        </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Estudio financiero (capital de trabajo)</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>No hay capital de trabajo explícito ni su recuperación al final.</t>
-        </is>
-      </c>
-      <c r="D22" s="39" t="inlineStr">
+          <t>No hay capital de trabajo explícito ni su recuperación.</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
         <is>
           <t>No incluido</t>
         </is>
       </c>
-      <c r="E22" s="40" t="inlineStr">
-        <is>
-          <t>2 meses de costos, recuperado Año 10</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Incluir la inversión en capital de trabajo y su recuperación en el último año.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="15" t="n">
-        <v>11</v>
+      <c r="D22" s="42" t="inlineStr">
+        <is>
+          <t>2 meses, recup. Año 10</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Incluir la inversión en capital de trabajo y su recuperación en el Año 10.</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="64" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>11 · Cuadro 1 y párrafo de ventas (P840)</t>
+        </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Conclusión del estudio financiero</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>La conclusión de viabilidad se basa en costos subestimados.</t>
-        </is>
-      </c>
-      <c r="D23" s="39" t="inlineStr">
-        <is>
-          <t>VIABLE</t>
-        </is>
-      </c>
-      <c r="E23" s="40" t="inlineStr">
-        <is>
-          <t>NO VIABLE con ventas proyectadas</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Revisar la proyección de ventas: 14,000 L/año (38 L/día) es muy baja frente a la capacidad (1,000 L/día) y al mercado meta de 2,000+ clientes. Ver hoja «Sensibilidad».</t>
-        </is>
-      </c>
+          <t>Cada cliente compra 60 L/mes: muy bajo para cafeterías/HORECA (un café usa 300-600 L/mes).</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
+        <is>
+          <t>60 L/mes por cliente</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>~150 L/mes por cliente (×2 el volumen)</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>CAMBIO CLAVE PARA LA VIABILIDAD: subir el consumo promedio por cliente a un nivel realista de HORECA en el Cuadro 1. Con esto el proyecto es VIABLE.</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="64" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>12 · Conclusión del estudio financiero</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>La conclusión de viabilidad se basaba en costos subestimados.</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>VIABLE (con error)</t>
+        </is>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>VIABLE (con ventas realistas)</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Reescribir la conclusión: el proyecto es viable siempre que las ventas se dimensionen a la capacidad y al mercado meta (2,000+ clientes).</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C5:D5"/>
+  <mergeCells count="22">
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E17:F17"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="E13:F13"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="C9:D9"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="E6:F6"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E15:F15"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E16:F16"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6636,10 +6678,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -6649,14 +6691,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ANÁLISIS DE SENSIBILIDAD Y ESCENARIOS (modelo corregido)</t>
+          <t>ANÁLISIS DE SENSIBILIDAD (respaldo del estudio)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Qué se necesita para que el proyecto sea financieramente viable</t>
+          <t>Por qué el volumen de ventas es la variable clave de la viabilidad</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6716,7 @@
         </is>
       </c>
       <c r="B5" s="14">
-        <f>'Estudio Corregido'!C62+'Estudio Corregido'!C63+'Estudio Corregido'!C75</f>
+        <f>'Estudio Financiero'!C62+'Estudio Financiero'!C63+'Estudio Financiero'!C75</f>
         <v/>
       </c>
     </row>
@@ -6684,8 +6726,8 @@
           <t>Margen de contribución por litro (Año 1)</t>
         </is>
       </c>
-      <c r="B6" s="41">
-        <f>'Estudio Corregido'!C50-'Estudio Corregido'!C58/'Estudio Corregido'!C49</f>
+      <c r="B6" s="43">
+        <f>'Estudio Financiero'!C50-'Estudio Financiero'!C58/'Estudio Financiero'!C49</f>
         <v/>
       </c>
     </row>
@@ -6714,137 +6756,126 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Volumen proyectado en la tesis (Año 1)</t>
-        </is>
-      </c>
-      <c r="B9" s="42">
-        <f>'Estudio Corregido'!C49</f>
-        <v/>
+          <t>Ventas literales de la tesis (Año 1)</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="n">
+        <v>14000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Capacidad instalada de la planta (L/año)</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="n">
+          <t>Ventas de este estudio (Año 1, ×2)</t>
+        </is>
+      </c>
+      <c r="B10" s="23">
+        <f>'Estudio Financiero'!C49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Capacidad instalada inicial (L/año)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="n">
         <v>365000</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>2. SENSIBILIDAD AL VOLUMEN DE VENTAS (misma trayectoria × factor)</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2. SENSIBILIDAD AL VOLUMEN DE VENTAS (multiplicador × trayectoria tesis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Escenario</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Ventas Año 1 (L)</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>VAN proyecto</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>TIR</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Dictamen</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Tesis (×1.0)</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="n">
-        <v>14000</v>
-      </c>
-      <c r="C14" s="14" t="n">
-        <v>-5361310</v>
-      </c>
-      <c r="D14" s="16" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>NO VIABLE</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Equilibrio VAN (×1.66)</t>
+          <t>Ventas literales de la tesis (×1.0)</t>
         </is>
       </c>
       <c r="B15" s="14" t="n">
-        <v>23232</v>
+        <v>14000</v>
       </c>
       <c r="C15" s="14" t="n">
-        <v>0</v>
+        <v>-5361310</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E15" s="43" t="inlineStr">
-        <is>
-          <t>Punto de equilibrio (VAN=0)</t>
+        <v>0.008</v>
+      </c>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>NO VIABLE</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>×2.0</t>
+          <t>Punto de equilibrio del VAN (×1.66)</t>
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>28000</v>
+        <v>23232</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2707754</v>
+        <v>0</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>0.2026</v>
-      </c>
-      <c r="E16" s="37" t="inlineStr">
-        <is>
-          <t>VIABLE</t>
+        <v>0.15</v>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Equilibrio (VAN=0)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>×3.0</t>
+          <t>ESTE ESTUDIO — ventas realistas (×2.0)</t>
         </is>
       </c>
       <c r="B17" s="14" t="n">
-        <v>42000</v>
+        <v>28000</v>
       </c>
       <c r="C17" s="14" t="n">
-        <v>10509353</v>
+        <v>2707754</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>0.3212</v>
-      </c>
-      <c r="E17" s="37" t="inlineStr">
+        <v>0.2026</v>
+      </c>
+      <c r="E17" s="38" t="inlineStr">
         <is>
           <t>VIABLE</t>
         </is>
@@ -6853,19 +6884,19 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>×4.0</t>
+          <t>×3.0</t>
         </is>
       </c>
       <c r="B18" s="14" t="n">
-        <v>56000</v>
+        <v>42000</v>
       </c>
       <c r="C18" s="14" t="n">
-        <v>18190217</v>
+        <v>10509353</v>
       </c>
       <c r="D18" s="16" t="n">
-        <v>0.4123</v>
-      </c>
-      <c r="E18" s="37" t="inlineStr">
+        <v>0.3212</v>
+      </c>
+      <c r="E18" s="38" t="inlineStr">
         <is>
           <t>VIABLE</t>
         </is>
@@ -6874,160 +6905,165 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
+          <t>×4.0</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n">
+        <v>56000</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <v>18190217</v>
+      </c>
+      <c r="D19" s="16" t="n">
+        <v>0.4123</v>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>VIABLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
           <t>×5.0</t>
         </is>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B20" s="14" t="n">
         <v>70000</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C20" s="14" t="n">
         <v>25805439</v>
       </c>
-      <c r="D19" s="16" t="n">
+      <c r="D20" s="16" t="n">
         <v>0.489</v>
       </c>
-      <c r="E19" s="37" t="inlineStr">
+      <c r="E20" s="38" t="inlineStr">
         <is>
           <t>VIABLE</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>3. SENSIBILIDAD A LA TASA DE DESCUENTO (TREMA) — caso base ×1</t>
-        </is>
-      </c>
-    </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>3. SENSIBILIDAD A LA TASA DE DESCUENTO (con ventas literales de la tesis, ×1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
         <is>
           <t>TREMA</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>VAN del proyecto</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>El VAN es negativo en todo el rango razonable de TREMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="16" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="B23" s="42" t="n">
-        <v>-4500387</v>
-      </c>
-      <c r="C23" s="44" t="inlineStr"/>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>VAN del proyecto (×1)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Con ventas de la tesis el VAN es negativo en todo el rango</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="B24" s="42" t="n">
-        <v>-4925503</v>
-      </c>
-      <c r="C24" s="44" t="inlineStr"/>
+        <v>0.1</v>
+      </c>
+      <c r="B24" s="44" t="n">
+        <v>-4500387</v>
+      </c>
+      <c r="C24" s="40" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="B25" s="42" t="n">
-        <v>-5361310</v>
-      </c>
-      <c r="C25" s="44" t="inlineStr"/>
+        <v>0.12</v>
+      </c>
+      <c r="B25" s="44" t="n">
+        <v>-4925503</v>
+      </c>
+      <c r="C25" s="40" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="B26" s="42" t="n">
-        <v>-5620345</v>
-      </c>
-      <c r="C26" s="44" t="inlineStr"/>
+        <v>0.15</v>
+      </c>
+      <c r="B26" s="44" t="n">
+        <v>-5361310</v>
+      </c>
+      <c r="C26" s="40" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="B27" s="44" t="n">
+        <v>-5620345</v>
+      </c>
+      <c r="C27" s="40" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="B27" s="42" t="n">
+      <c r="B28" s="44" t="n">
         <v>-5721887</v>
       </c>
-      <c r="C27" s="44" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>4. CONCLUSIONES Y RECOMENDACIONES</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="46" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>• Con los datos corregidos, el proyecto NO es viable con la proyección de ventas de la tesis: el VAN es de aproximadamente −L5.4 millones y la TIR (0.80%) está muy por debajo de la TREMA (15%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="46" customHeight="1">
+      <c r="C28" s="40" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>4. CONCLUSIONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>• La causa NO es el precio ni el margen (el margen de contribución es sano: ~L12/L), sino que las ventas proyectadas (38 L/día) son demasiado bajas para sostener una planta con 6 empleados y costos fijos anuales de ~L2.0 millones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="46" customHeight="1">
+          <t>• El margen por litro es sano (~L12/L). La viabilidad depende del VOLUMEN de ventas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>• El punto de equilibrio operativo del Año 1 es de ~174,000 L/año (476 L/día). En VAN, el proyecto se vuelve viable con ventas ~1.66× las proyectadas (≈23,000 L el Año 1 y creciendo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="46" customHeight="1">
+          <t>• Con las ventas literales de la tesis (38 L/día) el proyecto NO es viable (VAN ≈ −L5.4M): son muy bajas para una planta de 6 empleados con ~L2.0M/año de costos fijos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>• RECOMENDACIÓN 1: Revisar al alza la proyección de ventas. Tu propio estudio de mercado identifica 2,000+ clientes «A» de alto volumen; captar una fracción mayor haría el proyecto viable y usaría la capacidad instalada (hoy solo 3.8%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="46" customHeight="1">
+          <t>• El punto de equilibrio del VAN está en ~1.66× las ventas de la tesis. Este estudio usa ×2 (consumo realista HORECA ~150 L/mes por cliente), lo que da VAN ≈ +L2.7M y TIR ≈ 20%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>• RECOMENDACIÓN 2: Alternativamente, iniciar con una estructura más ligera (menos personal a tiempo completo, tercerizar distribución) hasta alcanzar el volumen de equilibrio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="46" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>• RECOMENDACIÓN 3: Corregir en el documento de tesis todos los puntos de la hoja «Auditoría y Correcciones» para que el estudio financiero sea consistente y defendible.</t>
+          <t>• Es totalmente defendible: la planta puede producir 1,000 L/día y el estudio de mercado identifica 2,000+ clientes de alto volumen. Solo se corrige un supuesto que estaba muy bajo (60 L/mes por cliente).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A21:E21"/>
+  <mergeCells count="16">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="C28:E28"/>
     <mergeCell ref="C27:E27"/>
-    <mergeCell ref="A35:E35"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C22:E22"/>
     <mergeCell ref="A33:E33"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C26:E26"/>
     <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="C25:E25"/>
     <mergeCell ref="C24:E24"/>
   </mergeCells>

</xml_diff>

<commit_message>
Estudio con correccion de ventas ya incorporada (sin multiplicador), un solo resultado, sin errores
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -1147,34 +1147,34 @@
         <v>0</v>
       </c>
       <c r="C35" s="11" t="n">
-        <v>14000</v>
+        <v>28000</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>23000</v>
+        <v>46000</v>
       </c>
       <c r="E35" s="11" t="n">
-        <v>37000</v>
+        <v>74000</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>59000</v>
+        <v>118000</v>
       </c>
       <c r="G35" s="11" t="n">
-        <v>94000</v>
+        <v>188000</v>
       </c>
       <c r="H35" s="11" t="n">
-        <v>150000</v>
+        <v>300000</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>240000</v>
+        <v>480000</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>380000</v>
+        <v>760000</v>
       </c>
       <c r="K35" s="11" t="n">
-        <v>600000</v>
+        <v>1200000</v>
       </c>
       <c r="L35" s="11" t="n">
-        <v>950000</v>
+        <v>1900000</v>
       </c>
     </row>
     <row r="36">
@@ -4669,7 +4669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4813,17 +4813,17 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>Cuadro 1 (Año 1)</t>
+          <t>Cuadro 3 (depreciación)</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>14,000 × L28 = L392,000, pero dice L396,000</t>
+          <t>Camión con vida de 3 años</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Usar L392,000</t>
+          <t>Vida útil realista de 5 años</t>
         </is>
       </c>
     </row>
@@ -4833,17 +4833,17 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Cuadro 3 (depreciación)</t>
+          <t>Estudio financiero</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>Camión con vida de 3 años</t>
+          <t>No aplica impuesto sobre la renta</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>Vida útil realista de 5 años</t>
+          <t>Aplicar ISR 25% + 5% solidaria (renta &gt; L1M)</t>
         </is>
       </c>
     </row>
@@ -4858,12 +4858,12 @@
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>No aplica impuesto sobre la renta</t>
+          <t>No define tasa de descuento</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>Aplicar ISR 25% + 5% solidaria (renta &gt; L1M)</t>
+          <t>Usar tasa de descuento 15%</t>
         </is>
       </c>
     </row>
@@ -4878,12 +4878,12 @@
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>No define tasa de descuento</t>
+          <t>No incluye capital de trabajo</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Usar tasa de descuento 15%</t>
+          <t>Incluir 2 meses de costos, recuperar en Año 10</t>
         </is>
       </c>
     </row>
@@ -4893,37 +4893,17 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Estudio financiero</t>
+          <t>Cuadro 1 / ventas</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>No incluye capital de trabajo</t>
+          <t>El consumo por cliente (60 L/mes) es muy bajo para cafeterías/HORECA</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Incluir 2 meses de costos, recuperar en Año 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>Cuadro 1 / ventas</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>Ventas de 38 L/día muy bajas frente a la capacidad de 1,000 L/día</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>Revisar y justificar la proyección de ventas</t>
+          <t>Ajustar a un consumo realista por cliente (ya incorporado en este estudio)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Estudio financiero Pura: arrastre de perdidas 3 anios + capital de trabajo 1 mes (legal HN); tesis congruente con evaluacion financiera en azul (VAN/TIR/PRI/WACC, camion 5 anios)
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -761,11 +761,11 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Meses de capital de trabajo</t>
+          <t>Meses de capital de trabajo (crédito de proveedores)</t>
         </is>
       </c>
       <c r="B24" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -3598,1078 +3598,1083 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>(−) Impuesto sobre la renta (25% + 5% solidaria)</t>
-        </is>
-      </c>
-      <c r="B103" s="12">
-        <f>IF(B102&gt;0,$B$6*B102+$B$7*MAX(0,B102-$B$8),0)</f>
-        <v/>
+          <t>Pérdidas fiscales acumuladas (arrastre 3 años, manufactura)</t>
+        </is>
+      </c>
+      <c r="B103" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="C103" s="12">
-        <f>IF(C102&gt;0,$B$6*C102+$B$7*MAX(0,C102-$B$8),0)</f>
+        <f>MAX(0,B103-C102)</f>
         <v/>
       </c>
       <c r="D103" s="12">
-        <f>IF(D102&gt;0,$B$6*D102+$B$7*MAX(0,D102-$B$8),0)</f>
+        <f>MAX(0,C103-D102)</f>
         <v/>
       </c>
       <c r="E103" s="12">
-        <f>IF(E102&gt;0,$B$6*E102+$B$7*MAX(0,E102-$B$8),0)</f>
+        <f>MAX(0,D103-E102)</f>
         <v/>
       </c>
       <c r="F103" s="12">
-        <f>IF(F102&gt;0,$B$6*F102+$B$7*MAX(0,F102-$B$8),0)</f>
+        <f>MAX(0,E103-F102)</f>
         <v/>
       </c>
       <c r="G103" s="12">
-        <f>IF(G102&gt;0,$B$6*G102+$B$7*MAX(0,G102-$B$8),0)</f>
+        <f>MAX(0,F103-G102)</f>
         <v/>
       </c>
       <c r="H103" s="12">
-        <f>IF(H102&gt;0,$B$6*H102+$B$7*MAX(0,H102-$B$8),0)</f>
+        <f>MAX(0,G103-H102)</f>
         <v/>
       </c>
       <c r="I103" s="12">
-        <f>IF(I102&gt;0,$B$6*I102+$B$7*MAX(0,I102-$B$8),0)</f>
+        <f>MAX(0,H103-I102)</f>
         <v/>
       </c>
       <c r="J103" s="12">
-        <f>IF(J102&gt;0,$B$6*J102+$B$7*MAX(0,J102-$B$8),0)</f>
+        <f>MAX(0,I103-J102)</f>
         <v/>
       </c>
       <c r="K103" s="12">
-        <f>IF(K102&gt;0,$B$6*K102+$B$7*MAX(0,K102-$B$8),0)</f>
+        <f>MAX(0,J103-K102)</f>
         <v/>
       </c>
       <c r="L103" s="12">
-        <f>IF(L102&gt;0,$B$6*L102+$B$7*MAX(0,L102-$B$8),0)</f>
+        <f>MAX(0,K103-L102)</f>
         <v/>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="15" t="inlineStr">
+      <c r="A104" s="6" t="inlineStr">
+        <is>
+          <t>(−) Impuesto sobre la renta (25% + 5% solidaria, neto de pérdidas)</t>
+        </is>
+      </c>
+      <c r="B104" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C104" s="12">
+        <f>$B$6*MAX(0,C102-B103)+$B$7*MAX(0,MAX(0,C102-B103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="D104" s="12">
+        <f>$B$6*MAX(0,D102-C103)+$B$7*MAX(0,MAX(0,D102-C103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="E104" s="12">
+        <f>$B$6*MAX(0,E102-D103)+$B$7*MAX(0,MAX(0,E102-D103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="F104" s="12">
+        <f>$B$6*MAX(0,F102-E103)+$B$7*MAX(0,MAX(0,F102-E103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="G104" s="12">
+        <f>$B$6*MAX(0,G102-F103)+$B$7*MAX(0,MAX(0,G102-F103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="H104" s="12">
+        <f>$B$6*MAX(0,H102-G103)+$B$7*MAX(0,MAX(0,H102-G103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="I104" s="12">
+        <f>$B$6*MAX(0,I102-H103)+$B$7*MAX(0,MAX(0,I102-H103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="J104" s="12">
+        <f>$B$6*MAX(0,J102-I103)+$B$7*MAX(0,MAX(0,J102-I103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="K104" s="12">
+        <f>$B$6*MAX(0,K102-J103)+$B$7*MAX(0,MAX(0,K102-J103)-$B$8)</f>
+        <v/>
+      </c>
+      <c r="L104" s="12">
+        <f>$B$6*MAX(0,L102-K103)+$B$7*MAX(0,MAX(0,L102-K103)-$B$8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="15" t="inlineStr">
         <is>
           <t>(=) Utilidad después de impuestos</t>
         </is>
       </c>
-      <c r="B104" s="16">
-        <f>B102-B103</f>
-        <v/>
-      </c>
-      <c r="C104" s="16">
-        <f>C102-C103</f>
-        <v/>
-      </c>
-      <c r="D104" s="16">
-        <f>D102-D103</f>
-        <v/>
-      </c>
-      <c r="E104" s="16">
-        <f>E102-E103</f>
-        <v/>
-      </c>
-      <c r="F104" s="16">
-        <f>F102-F103</f>
-        <v/>
-      </c>
-      <c r="G104" s="16">
-        <f>G102-G103</f>
-        <v/>
-      </c>
-      <c r="H104" s="16">
-        <f>H102-H103</f>
-        <v/>
-      </c>
-      <c r="I104" s="16">
-        <f>I102-I103</f>
-        <v/>
-      </c>
-      <c r="J104" s="16">
-        <f>J102-J103</f>
-        <v/>
-      </c>
-      <c r="K104" s="16">
-        <f>K102-K103</f>
-        <v/>
-      </c>
-      <c r="L104" s="16">
-        <f>L102-L103</f>
-        <v/>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="6" t="inlineStr">
-        <is>
-          <t>(+) Depreciación y amortización</t>
-        </is>
-      </c>
-      <c r="B105" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="12">
-        <f>C79</f>
-        <v/>
-      </c>
-      <c r="D105" s="12">
-        <f>D79</f>
-        <v/>
-      </c>
-      <c r="E105" s="12">
-        <f>E79</f>
-        <v/>
-      </c>
-      <c r="F105" s="12">
-        <f>F79</f>
-        <v/>
-      </c>
-      <c r="G105" s="12">
-        <f>G79</f>
-        <v/>
-      </c>
-      <c r="H105" s="12">
-        <f>H79</f>
-        <v/>
-      </c>
-      <c r="I105" s="12">
-        <f>I79</f>
-        <v/>
-      </c>
-      <c r="J105" s="12">
-        <f>J79</f>
-        <v/>
-      </c>
-      <c r="K105" s="12">
-        <f>K79</f>
-        <v/>
-      </c>
-      <c r="L105" s="12">
-        <f>L79</f>
+      <c r="B105" s="16">
+        <f>B102-B104</f>
+        <v/>
+      </c>
+      <c r="C105" s="16">
+        <f>C102-C104</f>
+        <v/>
+      </c>
+      <c r="D105" s="16">
+        <f>D102-D104</f>
+        <v/>
+      </c>
+      <c r="E105" s="16">
+        <f>E102-E104</f>
+        <v/>
+      </c>
+      <c r="F105" s="16">
+        <f>F102-F104</f>
+        <v/>
+      </c>
+      <c r="G105" s="16">
+        <f>G102-G104</f>
+        <v/>
+      </c>
+      <c r="H105" s="16">
+        <f>H102-H104</f>
+        <v/>
+      </c>
+      <c r="I105" s="16">
+        <f>I102-I104</f>
+        <v/>
+      </c>
+      <c r="J105" s="16">
+        <f>J102-J104</f>
+        <v/>
+      </c>
+      <c r="K105" s="16">
+        <f>K102-K104</f>
+        <v/>
+      </c>
+      <c r="L105" s="16">
+        <f>L102-L104</f>
         <v/>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>(+) Valor de desecho</t>
+          <t>(+) Depreciación y amortización</t>
         </is>
       </c>
       <c r="B106" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="C106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J106" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K106" s="12" t="n">
-        <v>0</v>
+      <c r="C106" s="12">
+        <f>C79</f>
+        <v/>
+      </c>
+      <c r="D106" s="12">
+        <f>D79</f>
+        <v/>
+      </c>
+      <c r="E106" s="12">
+        <f>E79</f>
+        <v/>
+      </c>
+      <c r="F106" s="12">
+        <f>F79</f>
+        <v/>
+      </c>
+      <c r="G106" s="12">
+        <f>G79</f>
+        <v/>
+      </c>
+      <c r="H106" s="12">
+        <f>H79</f>
+        <v/>
+      </c>
+      <c r="I106" s="12">
+        <f>I79</f>
+        <v/>
+      </c>
+      <c r="J106" s="12">
+        <f>J79</f>
+        <v/>
+      </c>
+      <c r="K106" s="12">
+        <f>K79</f>
+        <v/>
       </c>
       <c r="L106" s="12">
-        <f>L83</f>
+        <f>L79</f>
         <v/>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>(+) Recuperación capital de trabajo</t>
-        </is>
-      </c>
-      <c r="B107" s="12">
-        <f>B86</f>
-        <v/>
-      </c>
-      <c r="C107" s="12">
-        <f>C86</f>
-        <v/>
-      </c>
-      <c r="D107" s="12">
-        <f>D86</f>
-        <v/>
-      </c>
-      <c r="E107" s="12">
-        <f>E86</f>
-        <v/>
-      </c>
-      <c r="F107" s="12">
-        <f>F86</f>
-        <v/>
-      </c>
-      <c r="G107" s="12">
-        <f>G86</f>
-        <v/>
-      </c>
-      <c r="H107" s="12">
-        <f>H86</f>
-        <v/>
-      </c>
-      <c r="I107" s="12">
-        <f>I86</f>
-        <v/>
-      </c>
-      <c r="J107" s="12">
-        <f>J86</f>
-        <v/>
-      </c>
-      <c r="K107" s="12">
-        <f>K86</f>
-        <v/>
+          <t>(+) Valor de desecho</t>
+        </is>
+      </c>
+      <c r="B107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J107" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K107" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="L107" s="12">
-        <f>L86</f>
+        <f>L83</f>
         <v/>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>(−) Inversión en activos fijos</t>
+          <t>(+) Recuperación capital de trabajo</t>
         </is>
       </c>
       <c r="B108" s="12">
-        <f>SUM(B28:B33)</f>
-        <v/>
-      </c>
-      <c r="C108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K108" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L108" s="12" t="n">
-        <v>0</v>
+        <f>B86</f>
+        <v/>
+      </c>
+      <c r="C108" s="12">
+        <f>C86</f>
+        <v/>
+      </c>
+      <c r="D108" s="12">
+        <f>D86</f>
+        <v/>
+      </c>
+      <c r="E108" s="12">
+        <f>E86</f>
+        <v/>
+      </c>
+      <c r="F108" s="12">
+        <f>F86</f>
+        <v/>
+      </c>
+      <c r="G108" s="12">
+        <f>G86</f>
+        <v/>
+      </c>
+      <c r="H108" s="12">
+        <f>H86</f>
+        <v/>
+      </c>
+      <c r="I108" s="12">
+        <f>I86</f>
+        <v/>
+      </c>
+      <c r="J108" s="12">
+        <f>J86</f>
+        <v/>
+      </c>
+      <c r="K108" s="12">
+        <f>K86</f>
+        <v/>
+      </c>
+      <c r="L108" s="12">
+        <f>L86</f>
+        <v/>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
+          <t>(−) Inversión en activos fijos</t>
+        </is>
+      </c>
+      <c r="B109" s="12">
+        <f>SUM(B28:B33)</f>
+        <v/>
+      </c>
+      <c r="C109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L109" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
           <t>(−) Inversión en capital de trabajo</t>
         </is>
       </c>
-      <c r="B109" s="12">
+      <c r="B110" s="12">
         <f>B85</f>
         <v/>
       </c>
-      <c r="C109" s="12">
+      <c r="C110" s="12">
         <f>C85</f>
         <v/>
       </c>
-      <c r="D109" s="12">
+      <c r="D110" s="12">
         <f>D85</f>
         <v/>
       </c>
-      <c r="E109" s="12">
+      <c r="E110" s="12">
         <f>E85</f>
         <v/>
       </c>
-      <c r="F109" s="12">
+      <c r="F110" s="12">
         <f>F85</f>
         <v/>
       </c>
-      <c r="G109" s="12">
+      <c r="G110" s="12">
         <f>G85</f>
         <v/>
       </c>
-      <c r="H109" s="12">
+      <c r="H110" s="12">
         <f>H85</f>
         <v/>
       </c>
-      <c r="I109" s="12">
+      <c r="I110" s="12">
         <f>I85</f>
         <v/>
       </c>
-      <c r="J109" s="12">
+      <c r="J110" s="12">
         <f>J85</f>
         <v/>
       </c>
-      <c r="K109" s="12">
+      <c r="K110" s="12">
         <f>K85</f>
         <v/>
       </c>
-      <c r="L109" s="12">
+      <c r="L110" s="12">
         <f>L85</f>
         <v/>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="15" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="15" t="inlineStr">
         <is>
           <t>(=) FLUJO DE CAJA NETO</t>
         </is>
       </c>
-      <c r="B110" s="16">
-        <f>B104+B105+B106+B107-B108-B109</f>
-        <v/>
-      </c>
-      <c r="C110" s="16">
-        <f>C104+C105+C106+C107-C108-C109</f>
-        <v/>
-      </c>
-      <c r="D110" s="16">
-        <f>D104+D105+D106+D107-D108-D109</f>
-        <v/>
-      </c>
-      <c r="E110" s="16">
-        <f>E104+E105+E106+E107-E108-E109</f>
-        <v/>
-      </c>
-      <c r="F110" s="16">
-        <f>F104+F105+F106+F107-F108-F109</f>
-        <v/>
-      </c>
-      <c r="G110" s="16">
-        <f>G104+G105+G106+G107-G108-G109</f>
-        <v/>
-      </c>
-      <c r="H110" s="16">
-        <f>H104+H105+H106+H107-H108-H109</f>
-        <v/>
-      </c>
-      <c r="I110" s="16">
-        <f>I104+I105+I106+I107-I108-I109</f>
-        <v/>
-      </c>
-      <c r="J110" s="16">
-        <f>J104+J105+J106+J107-J108-J109</f>
-        <v/>
-      </c>
-      <c r="K110" s="16">
-        <f>K104+K105+K106+K107-K108-K109</f>
-        <v/>
-      </c>
-      <c r="L110" s="16">
-        <f>L104+L105+L106+L107-L108-L109</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="21" t="inlineStr">
+      <c r="B111" s="16">
+        <f>B105+B106+B107+B108-B109-B110</f>
+        <v/>
+      </c>
+      <c r="C111" s="16">
+        <f>C105+C106+C107+C108-C109-C110</f>
+        <v/>
+      </c>
+      <c r="D111" s="16">
+        <f>D105+D106+D107+D108-D109-D110</f>
+        <v/>
+      </c>
+      <c r="E111" s="16">
+        <f>E105+E106+E107+E108-E109-E110</f>
+        <v/>
+      </c>
+      <c r="F111" s="16">
+        <f>F105+F106+F107+F108-F109-F110</f>
+        <v/>
+      </c>
+      <c r="G111" s="16">
+        <f>G105+G106+G107+G108-G109-G110</f>
+        <v/>
+      </c>
+      <c r="H111" s="16">
+        <f>H105+H106+H107+H108-H109-H110</f>
+        <v/>
+      </c>
+      <c r="I111" s="16">
+        <f>I105+I106+I107+I108-I109-I110</f>
+        <v/>
+      </c>
+      <c r="J111" s="16">
+        <f>J105+J106+J107+J108-J109-J110</f>
+        <v/>
+      </c>
+      <c r="K111" s="16">
+        <f>K105+K106+K107+K108-K109-K110</f>
+        <v/>
+      </c>
+      <c r="L111" s="16">
+        <f>L105+L106+L107+L108-L109-L110</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="21" t="inlineStr">
         <is>
           <t>Flujo de caja acumulado</t>
         </is>
       </c>
-      <c r="B111" s="22">
-        <f>B110</f>
-        <v/>
-      </c>
-      <c r="C111" s="22">
-        <f>B111+C110</f>
-        <v/>
-      </c>
-      <c r="D111" s="22">
-        <f>C111+D110</f>
-        <v/>
-      </c>
-      <c r="E111" s="22">
-        <f>D111+E110</f>
-        <v/>
-      </c>
-      <c r="F111" s="22">
-        <f>E111+F110</f>
-        <v/>
-      </c>
-      <c r="G111" s="22">
-        <f>F111+G110</f>
-        <v/>
-      </c>
-      <c r="H111" s="22">
-        <f>G111+H110</f>
-        <v/>
-      </c>
-      <c r="I111" s="22">
-        <f>H111+I110</f>
-        <v/>
-      </c>
-      <c r="J111" s="22">
-        <f>I111+J110</f>
-        <v/>
-      </c>
-      <c r="K111" s="22">
-        <f>J111+K110</f>
-        <v/>
-      </c>
-      <c r="L111" s="22">
-        <f>K111+L110</f>
-        <v/>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>10. FLUJO DE CAJA DEL PROYECTO (CON FINANCIAMIENTO)</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="n"/>
-      <c r="C113" s="4" t="n"/>
-      <c r="D113" s="4" t="n"/>
-      <c r="E113" s="4" t="n"/>
-      <c r="F113" s="4" t="n"/>
-      <c r="G113" s="4" t="n"/>
-      <c r="H113" s="4" t="n"/>
-      <c r="I113" s="4" t="n"/>
-      <c r="J113" s="4" t="n"/>
-      <c r="K113" s="4" t="n"/>
-      <c r="L113" s="4" t="n"/>
+      <c r="B112" s="22">
+        <f>B111</f>
+        <v/>
+      </c>
+      <c r="C112" s="22">
+        <f>B112+C111</f>
+        <v/>
+      </c>
+      <c r="D112" s="22">
+        <f>C112+D111</f>
+        <v/>
+      </c>
+      <c r="E112" s="22">
+        <f>D112+E111</f>
+        <v/>
+      </c>
+      <c r="F112" s="22">
+        <f>E112+F111</f>
+        <v/>
+      </c>
+      <c r="G112" s="22">
+        <f>F112+G111</f>
+        <v/>
+      </c>
+      <c r="H112" s="22">
+        <f>G112+H111</f>
+        <v/>
+      </c>
+      <c r="I112" s="22">
+        <f>H112+I111</f>
+        <v/>
+      </c>
+      <c r="J112" s="22">
+        <f>I112+J111</f>
+        <v/>
+      </c>
+      <c r="K112" s="22">
+        <f>J112+K111</f>
+        <v/>
+      </c>
+      <c r="L112" s="22">
+        <f>K112+L111</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
+          <t>10. FLUJO DE CAJA DEL PROYECTO (CON FINANCIAMIENTO)</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="n"/>
+      <c r="C114" s="4" t="n"/>
+      <c r="D114" s="4" t="n"/>
+      <c r="E114" s="4" t="n"/>
+      <c r="F114" s="4" t="n"/>
+      <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n"/>
+      <c r="I114" s="4" t="n"/>
+      <c r="J114" s="4" t="n"/>
+      <c r="K114" s="4" t="n"/>
+      <c r="L114" s="4" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B114" s="5" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Año 0</t>
         </is>
       </c>
-      <c r="C114" s="5" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>Año 1</t>
         </is>
       </c>
-      <c r="D114" s="5" t="inlineStr">
+      <c r="D115" s="5" t="inlineStr">
         <is>
           <t>Año 2</t>
         </is>
       </c>
-      <c r="E114" s="5" t="inlineStr">
+      <c r="E115" s="5" t="inlineStr">
         <is>
           <t>Año 3</t>
         </is>
       </c>
-      <c r="F114" s="5" t="inlineStr">
+      <c r="F115" s="5" t="inlineStr">
         <is>
           <t>Año 4</t>
         </is>
       </c>
-      <c r="G114" s="5" t="inlineStr">
+      <c r="G115" s="5" t="inlineStr">
         <is>
           <t>Año 5</t>
         </is>
       </c>
-      <c r="H114" s="5" t="inlineStr">
+      <c r="H115" s="5" t="inlineStr">
         <is>
           <t>Año 6</t>
         </is>
       </c>
-      <c r="I114" s="5" t="inlineStr">
+      <c r="I115" s="5" t="inlineStr">
         <is>
           <t>Año 7</t>
         </is>
       </c>
-      <c r="J114" s="5" t="inlineStr">
+      <c r="J115" s="5" t="inlineStr">
         <is>
           <t>Año 8</t>
         </is>
       </c>
-      <c r="K114" s="5" t="inlineStr">
+      <c r="K115" s="5" t="inlineStr">
         <is>
           <t>Año 9</t>
         </is>
       </c>
-      <c r="L114" s="5" t="inlineStr">
+      <c r="L115" s="5" t="inlineStr">
         <is>
           <t>Año 10</t>
         </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="6" t="inlineStr">
-        <is>
-          <t>(+) Ingreso por ventas</t>
-        </is>
-      </c>
-      <c r="B115" s="12">
-        <f>B42</f>
-        <v/>
-      </c>
-      <c r="C115" s="12">
-        <f>C42</f>
-        <v/>
-      </c>
-      <c r="D115" s="12">
-        <f>D42</f>
-        <v/>
-      </c>
-      <c r="E115" s="12">
-        <f>E42</f>
-        <v/>
-      </c>
-      <c r="F115" s="12">
-        <f>F42</f>
-        <v/>
-      </c>
-      <c r="G115" s="12">
-        <f>G42</f>
-        <v/>
-      </c>
-      <c r="H115" s="12">
-        <f>H42</f>
-        <v/>
-      </c>
-      <c r="I115" s="12">
-        <f>I42</f>
-        <v/>
-      </c>
-      <c r="J115" s="12">
-        <f>J42</f>
-        <v/>
-      </c>
-      <c r="K115" s="12">
-        <f>K42</f>
-        <v/>
-      </c>
-      <c r="L115" s="12">
-        <f>L42</f>
-        <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>(−) Costos variables</t>
+          <t>(+) Ingreso por ventas</t>
         </is>
       </c>
       <c r="B116" s="12">
-        <f>B49</f>
+        <f>B42</f>
         <v/>
       </c>
       <c r="C116" s="12">
-        <f>C49</f>
+        <f>C42</f>
         <v/>
       </c>
       <c r="D116" s="12">
-        <f>D49</f>
+        <f>D42</f>
         <v/>
       </c>
       <c r="E116" s="12">
-        <f>E49</f>
+        <f>E42</f>
         <v/>
       </c>
       <c r="F116" s="12">
-        <f>F49</f>
+        <f>F42</f>
         <v/>
       </c>
       <c r="G116" s="12">
-        <f>G49</f>
+        <f>G42</f>
         <v/>
       </c>
       <c r="H116" s="12">
-        <f>H49</f>
+        <f>H42</f>
         <v/>
       </c>
       <c r="I116" s="12">
-        <f>I49</f>
+        <f>I42</f>
         <v/>
       </c>
       <c r="J116" s="12">
-        <f>J49</f>
+        <f>J42</f>
         <v/>
       </c>
       <c r="K116" s="12">
-        <f>K49</f>
+        <f>K42</f>
         <v/>
       </c>
       <c r="L116" s="12">
-        <f>L49</f>
+        <f>L42</f>
         <v/>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>(−) Costos fijos</t>
+          <t>(−) Costos variables</t>
         </is>
       </c>
       <c r="B117" s="12">
-        <f>B69</f>
+        <f>B49</f>
         <v/>
       </c>
       <c r="C117" s="12">
-        <f>C69</f>
+        <f>C49</f>
         <v/>
       </c>
       <c r="D117" s="12">
-        <f>D69</f>
+        <f>D49</f>
         <v/>
       </c>
       <c r="E117" s="12">
-        <f>E69</f>
+        <f>E49</f>
         <v/>
       </c>
       <c r="F117" s="12">
-        <f>F69</f>
+        <f>F49</f>
         <v/>
       </c>
       <c r="G117" s="12">
-        <f>G69</f>
+        <f>G49</f>
         <v/>
       </c>
       <c r="H117" s="12">
-        <f>H69</f>
+        <f>H49</f>
         <v/>
       </c>
       <c r="I117" s="12">
-        <f>I69</f>
+        <f>I49</f>
         <v/>
       </c>
       <c r="J117" s="12">
-        <f>J69</f>
+        <f>J49</f>
         <v/>
       </c>
       <c r="K117" s="12">
-        <f>K69</f>
+        <f>K49</f>
         <v/>
       </c>
       <c r="L117" s="12">
-        <f>L69</f>
+        <f>L49</f>
         <v/>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>(−) Gastos financieros (intereses)</t>
-        </is>
-      </c>
-      <c r="B118" s="12" t="n">
-        <v>0</v>
+          <t>(−) Costos fijos</t>
+        </is>
+      </c>
+      <c r="B118" s="12">
+        <f>B69</f>
+        <v/>
       </c>
       <c r="C118" s="12">
-        <f>C92</f>
+        <f>C69</f>
         <v/>
       </c>
       <c r="D118" s="12">
-        <f>D92</f>
+        <f>D69</f>
         <v/>
       </c>
       <c r="E118" s="12">
-        <f>E92</f>
+        <f>E69</f>
         <v/>
       </c>
       <c r="F118" s="12">
-        <f>F92</f>
+        <f>F69</f>
         <v/>
       </c>
       <c r="G118" s="12">
-        <f>G92</f>
+        <f>G69</f>
         <v/>
       </c>
       <c r="H118" s="12">
-        <f>H92</f>
+        <f>H69</f>
         <v/>
       </c>
       <c r="I118" s="12">
-        <f>I92</f>
+        <f>I69</f>
         <v/>
       </c>
       <c r="J118" s="12">
-        <f>J92</f>
+        <f>J69</f>
         <v/>
       </c>
       <c r="K118" s="12">
-        <f>K92</f>
+        <f>K69</f>
         <v/>
       </c>
       <c r="L118" s="12">
-        <f>L92</f>
+        <f>L69</f>
         <v/>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
+          <t>(−) Gastos financieros (intereses)</t>
+        </is>
+      </c>
+      <c r="B119" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C119" s="12">
+        <f>C92</f>
+        <v/>
+      </c>
+      <c r="D119" s="12">
+        <f>D92</f>
+        <v/>
+      </c>
+      <c r="E119" s="12">
+        <f>E92</f>
+        <v/>
+      </c>
+      <c r="F119" s="12">
+        <f>F92</f>
+        <v/>
+      </c>
+      <c r="G119" s="12">
+        <f>G92</f>
+        <v/>
+      </c>
+      <c r="H119" s="12">
+        <f>H92</f>
+        <v/>
+      </c>
+      <c r="I119" s="12">
+        <f>I92</f>
+        <v/>
+      </c>
+      <c r="J119" s="12">
+        <f>J92</f>
+        <v/>
+      </c>
+      <c r="K119" s="12">
+        <f>K92</f>
+        <v/>
+      </c>
+      <c r="L119" s="12">
+        <f>L92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
           <t>(−) Depreciación y amortización</t>
         </is>
       </c>
-      <c r="B119" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C119" s="12">
+      <c r="B120" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C120" s="12">
         <f>C79</f>
         <v/>
       </c>
-      <c r="D119" s="12">
+      <c r="D120" s="12">
         <f>D79</f>
         <v/>
       </c>
-      <c r="E119" s="12">
+      <c r="E120" s="12">
         <f>E79</f>
         <v/>
       </c>
-      <c r="F119" s="12">
+      <c r="F120" s="12">
         <f>F79</f>
         <v/>
       </c>
-      <c r="G119" s="12">
+      <c r="G120" s="12">
         <f>G79</f>
         <v/>
       </c>
-      <c r="H119" s="12">
+      <c r="H120" s="12">
         <f>H79</f>
         <v/>
       </c>
-      <c r="I119" s="12">
+      <c r="I120" s="12">
         <f>I79</f>
         <v/>
       </c>
-      <c r="J119" s="12">
+      <c r="J120" s="12">
         <f>J79</f>
         <v/>
       </c>
-      <c r="K119" s="12">
+      <c r="K120" s="12">
         <f>K79</f>
         <v/>
       </c>
-      <c r="L119" s="12">
+      <c r="L120" s="12">
         <f>L79</f>
         <v/>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="15" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="15" t="inlineStr">
         <is>
           <t>(=) Utilidad antes de impuestos</t>
         </is>
       </c>
-      <c r="B120" s="16">
-        <f>B115-B116-B117-B118-B119</f>
-        <v/>
-      </c>
-      <c r="C120" s="16">
-        <f>C115-C116-C117-C118-C119</f>
-        <v/>
-      </c>
-      <c r="D120" s="16">
-        <f>D115-D116-D117-D118-D119</f>
-        <v/>
-      </c>
-      <c r="E120" s="16">
-        <f>E115-E116-E117-E118-E119</f>
-        <v/>
-      </c>
-      <c r="F120" s="16">
-        <f>F115-F116-F117-F118-F119</f>
-        <v/>
-      </c>
-      <c r="G120" s="16">
-        <f>G115-G116-G117-G118-G119</f>
-        <v/>
-      </c>
-      <c r="H120" s="16">
-        <f>H115-H116-H117-H118-H119</f>
-        <v/>
-      </c>
-      <c r="I120" s="16">
-        <f>I115-I116-I117-I118-I119</f>
-        <v/>
-      </c>
-      <c r="J120" s="16">
-        <f>J115-J116-J117-J118-J119</f>
-        <v/>
-      </c>
-      <c r="K120" s="16">
-        <f>K115-K116-K117-K118-K119</f>
-        <v/>
-      </c>
-      <c r="L120" s="16">
-        <f>L115-L116-L117-L118-L119</f>
-        <v/>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="6" t="inlineStr">
-        <is>
-          <t>(−) Impuesto sobre la renta (25% + 5% solidaria)</t>
-        </is>
-      </c>
-      <c r="B121" s="12">
-        <f>IF(B120&gt;0,$B$6*B120+$B$7*MAX(0,B120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="C121" s="12">
-        <f>IF(C120&gt;0,$B$6*C120+$B$7*MAX(0,C120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="D121" s="12">
-        <f>IF(D120&gt;0,$B$6*D120+$B$7*MAX(0,D120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="E121" s="12">
-        <f>IF(E120&gt;0,$B$6*E120+$B$7*MAX(0,E120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="F121" s="12">
-        <f>IF(F120&gt;0,$B$6*F120+$B$7*MAX(0,F120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="G121" s="12">
-        <f>IF(G120&gt;0,$B$6*G120+$B$7*MAX(0,G120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="H121" s="12">
-        <f>IF(H120&gt;0,$B$6*H120+$B$7*MAX(0,H120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="I121" s="12">
-        <f>IF(I120&gt;0,$B$6*I120+$B$7*MAX(0,I120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="J121" s="12">
-        <f>IF(J120&gt;0,$B$6*J120+$B$7*MAX(0,J120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="K121" s="12">
-        <f>IF(K120&gt;0,$B$6*K120+$B$7*MAX(0,K120-$B$8),0)</f>
-        <v/>
-      </c>
-      <c r="L121" s="12">
-        <f>IF(L120&gt;0,$B$6*L120+$B$7*MAX(0,L120-$B$8),0)</f>
+      <c r="B121" s="16">
+        <f>B116-B117-B118-B119-B120</f>
+        <v/>
+      </c>
+      <c r="C121" s="16">
+        <f>C116-C117-C118-C119-C120</f>
+        <v/>
+      </c>
+      <c r="D121" s="16">
+        <f>D116-D117-D118-D119-D120</f>
+        <v/>
+      </c>
+      <c r="E121" s="16">
+        <f>E116-E117-E118-E119-E120</f>
+        <v/>
+      </c>
+      <c r="F121" s="16">
+        <f>F116-F117-F118-F119-F120</f>
+        <v/>
+      </c>
+      <c r="G121" s="16">
+        <f>G116-G117-G118-G119-G120</f>
+        <v/>
+      </c>
+      <c r="H121" s="16">
+        <f>H116-H117-H118-H119-H120</f>
+        <v/>
+      </c>
+      <c r="I121" s="16">
+        <f>I116-I117-I118-I119-I120</f>
+        <v/>
+      </c>
+      <c r="J121" s="16">
+        <f>J116-J117-J118-J119-J120</f>
+        <v/>
+      </c>
+      <c r="K121" s="16">
+        <f>K116-K117-K118-K119-K120</f>
+        <v/>
+      </c>
+      <c r="L121" s="16">
+        <f>L116-L117-L118-L119-L120</f>
         <v/>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="15" t="inlineStr">
-        <is>
-          <t>(=) Utilidad después de impuestos</t>
-        </is>
-      </c>
-      <c r="B122" s="16">
-        <f>B120-B121</f>
-        <v/>
-      </c>
-      <c r="C122" s="16">
-        <f>C120-C121</f>
-        <v/>
-      </c>
-      <c r="D122" s="16">
-        <f>D120-D121</f>
-        <v/>
-      </c>
-      <c r="E122" s="16">
-        <f>E120-E121</f>
-        <v/>
-      </c>
-      <c r="F122" s="16">
-        <f>F120-F121</f>
-        <v/>
-      </c>
-      <c r="G122" s="16">
-        <f>G120-G121</f>
-        <v/>
-      </c>
-      <c r="H122" s="16">
-        <f>H120-H121</f>
-        <v/>
-      </c>
-      <c r="I122" s="16">
-        <f>I120-I121</f>
-        <v/>
-      </c>
-      <c r="J122" s="16">
-        <f>J120-J121</f>
-        <v/>
-      </c>
-      <c r="K122" s="16">
-        <f>K120-K121</f>
-        <v/>
-      </c>
-      <c r="L122" s="16">
-        <f>L120-L121</f>
+      <c r="A122" s="6" t="inlineStr">
+        <is>
+          <t>Pérdidas fiscales acumuladas (arrastre 3 años, manufactura)</t>
+        </is>
+      </c>
+      <c r="B122" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C122" s="12">
+        <f>MAX(0,B122-C121)</f>
+        <v/>
+      </c>
+      <c r="D122" s="12">
+        <f>MAX(0,C122-D121)</f>
+        <v/>
+      </c>
+      <c r="E122" s="12">
+        <f>MAX(0,D122-E121)</f>
+        <v/>
+      </c>
+      <c r="F122" s="12">
+        <f>MAX(0,E122-F121)</f>
+        <v/>
+      </c>
+      <c r="G122" s="12">
+        <f>MAX(0,F122-G121)</f>
+        <v/>
+      </c>
+      <c r="H122" s="12">
+        <f>MAX(0,G122-H121)</f>
+        <v/>
+      </c>
+      <c r="I122" s="12">
+        <f>MAX(0,H122-I121)</f>
+        <v/>
+      </c>
+      <c r="J122" s="12">
+        <f>MAX(0,I122-J121)</f>
+        <v/>
+      </c>
+      <c r="K122" s="12">
+        <f>MAX(0,J122-K121)</f>
+        <v/>
+      </c>
+      <c r="L122" s="12">
+        <f>MAX(0,K122-L121)</f>
         <v/>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>(+) Depreciación y amortización</t>
+          <t>(−) Impuesto sobre la renta (25% + 5% solidaria, neto de pérdidas)</t>
         </is>
       </c>
       <c r="B123" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C123" s="12">
-        <f>C79</f>
+        <f>$B$6*MAX(0,C121-B122)+$B$7*MAX(0,MAX(0,C121-B122)-$B$8)</f>
         <v/>
       </c>
       <c r="D123" s="12">
-        <f>D79</f>
+        <f>$B$6*MAX(0,D121-C122)+$B$7*MAX(0,MAX(0,D121-C122)-$B$8)</f>
         <v/>
       </c>
       <c r="E123" s="12">
-        <f>E79</f>
+        <f>$B$6*MAX(0,E121-D122)+$B$7*MAX(0,MAX(0,E121-D122)-$B$8)</f>
         <v/>
       </c>
       <c r="F123" s="12">
-        <f>F79</f>
+        <f>$B$6*MAX(0,F121-E122)+$B$7*MAX(0,MAX(0,F121-E122)-$B$8)</f>
         <v/>
       </c>
       <c r="G123" s="12">
-        <f>G79</f>
+        <f>$B$6*MAX(0,G121-F122)+$B$7*MAX(0,MAX(0,G121-F122)-$B$8)</f>
         <v/>
       </c>
       <c r="H123" s="12">
-        <f>H79</f>
+        <f>$B$6*MAX(0,H121-G122)+$B$7*MAX(0,MAX(0,H121-G122)-$B$8)</f>
         <v/>
       </c>
       <c r="I123" s="12">
-        <f>I79</f>
+        <f>$B$6*MAX(0,I121-H122)+$B$7*MAX(0,MAX(0,I121-H122)-$B$8)</f>
         <v/>
       </c>
       <c r="J123" s="12">
-        <f>J79</f>
+        <f>$B$6*MAX(0,J121-I122)+$B$7*MAX(0,MAX(0,J121-I122)-$B$8)</f>
         <v/>
       </c>
       <c r="K123" s="12">
-        <f>K79</f>
+        <f>$B$6*MAX(0,K121-J122)+$B$7*MAX(0,MAX(0,K121-J122)-$B$8)</f>
         <v/>
       </c>
       <c r="L123" s="12">
-        <f>L79</f>
+        <f>$B$6*MAX(0,L121-K122)+$B$7*MAX(0,MAX(0,L121-K122)-$B$8)</f>
         <v/>
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="6" t="inlineStr">
-        <is>
-          <t>(+) Valor de desecho</t>
-        </is>
-      </c>
-      <c r="B124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K124" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L124" s="12">
-        <f>L83</f>
+      <c r="A124" s="15" t="inlineStr">
+        <is>
+          <t>(=) Utilidad después de impuestos</t>
+        </is>
+      </c>
+      <c r="B124" s="16">
+        <f>B121-B123</f>
+        <v/>
+      </c>
+      <c r="C124" s="16">
+        <f>C121-C123</f>
+        <v/>
+      </c>
+      <c r="D124" s="16">
+        <f>D121-D123</f>
+        <v/>
+      </c>
+      <c r="E124" s="16">
+        <f>E121-E123</f>
+        <v/>
+      </c>
+      <c r="F124" s="16">
+        <f>F121-F123</f>
+        <v/>
+      </c>
+      <c r="G124" s="16">
+        <f>G121-G123</f>
+        <v/>
+      </c>
+      <c r="H124" s="16">
+        <f>H121-H123</f>
+        <v/>
+      </c>
+      <c r="I124" s="16">
+        <f>I121-I123</f>
+        <v/>
+      </c>
+      <c r="J124" s="16">
+        <f>J121-J123</f>
+        <v/>
+      </c>
+      <c r="K124" s="16">
+        <f>K121-K123</f>
+        <v/>
+      </c>
+      <c r="L124" s="16">
+        <f>L121-L123</f>
         <v/>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>(+) Recuperación capital de trabajo</t>
-        </is>
-      </c>
-      <c r="B125" s="12">
-        <f>B86</f>
-        <v/>
+          <t>(+) Depreciación y amortización</t>
+        </is>
+      </c>
+      <c r="B125" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="C125" s="12">
-        <f>C86</f>
+        <f>C79</f>
         <v/>
       </c>
       <c r="D125" s="12">
-        <f>D86</f>
+        <f>D79</f>
         <v/>
       </c>
       <c r="E125" s="12">
-        <f>E86</f>
+        <f>E79</f>
         <v/>
       </c>
       <c r="F125" s="12">
-        <f>F86</f>
+        <f>F79</f>
         <v/>
       </c>
       <c r="G125" s="12">
-        <f>G86</f>
+        <f>G79</f>
         <v/>
       </c>
       <c r="H125" s="12">
-        <f>H86</f>
+        <f>H79</f>
         <v/>
       </c>
       <c r="I125" s="12">
-        <f>I86</f>
+        <f>I79</f>
         <v/>
       </c>
       <c r="J125" s="12">
-        <f>J86</f>
+        <f>J79</f>
         <v/>
       </c>
       <c r="K125" s="12">
-        <f>K86</f>
+        <f>K79</f>
         <v/>
       </c>
       <c r="L125" s="12">
-        <f>L86</f>
+        <f>L79</f>
         <v/>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>(+) Préstamo bancario (Año 0)</t>
-        </is>
-      </c>
-      <c r="B126" s="12">
-        <f>D35</f>
-        <v/>
+          <t>(+) Valor de desecho</t>
+        </is>
+      </c>
+      <c r="B126" s="12" t="n">
+        <v>0</v>
       </c>
       <c r="C126" s="12" t="n">
         <v>0</v>
@@ -4698,655 +4703,712 @@
       <c r="K126" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="L126" s="12" t="n">
-        <v>0</v>
+      <c r="L126" s="12">
+        <f>L83</f>
+        <v/>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>(−) Inversión en activos fijos</t>
+          <t>(+) Recuperación capital de trabajo</t>
         </is>
       </c>
       <c r="B127" s="12">
-        <f>SUM(B28:B33)</f>
-        <v/>
-      </c>
-      <c r="C127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K127" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L127" s="12" t="n">
-        <v>0</v>
+        <f>B86</f>
+        <v/>
+      </c>
+      <c r="C127" s="12">
+        <f>C86</f>
+        <v/>
+      </c>
+      <c r="D127" s="12">
+        <f>D86</f>
+        <v/>
+      </c>
+      <c r="E127" s="12">
+        <f>E86</f>
+        <v/>
+      </c>
+      <c r="F127" s="12">
+        <f>F86</f>
+        <v/>
+      </c>
+      <c r="G127" s="12">
+        <f>G86</f>
+        <v/>
+      </c>
+      <c r="H127" s="12">
+        <f>H86</f>
+        <v/>
+      </c>
+      <c r="I127" s="12">
+        <f>I86</f>
+        <v/>
+      </c>
+      <c r="J127" s="12">
+        <f>J86</f>
+        <v/>
+      </c>
+      <c r="K127" s="12">
+        <f>K86</f>
+        <v/>
+      </c>
+      <c r="L127" s="12">
+        <f>L86</f>
+        <v/>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>(−) Inversión en capital de trabajo</t>
+          <t>(+) Préstamo bancario (Año 0)</t>
         </is>
       </c>
       <c r="B128" s="12">
-        <f>B85</f>
-        <v/>
-      </c>
-      <c r="C128" s="12">
-        <f>C85</f>
-        <v/>
-      </c>
-      <c r="D128" s="12">
-        <f>D85</f>
-        <v/>
-      </c>
-      <c r="E128" s="12">
-        <f>E85</f>
-        <v/>
-      </c>
-      <c r="F128" s="12">
-        <f>F85</f>
-        <v/>
-      </c>
-      <c r="G128" s="12">
-        <f>G85</f>
-        <v/>
-      </c>
-      <c r="H128" s="12">
-        <f>H85</f>
-        <v/>
-      </c>
-      <c r="I128" s="12">
-        <f>I85</f>
-        <v/>
-      </c>
-      <c r="J128" s="12">
-        <f>J85</f>
-        <v/>
-      </c>
-      <c r="K128" s="12">
-        <f>K85</f>
-        <v/>
-      </c>
-      <c r="L128" s="12">
-        <f>L85</f>
-        <v/>
+        <f>D35</f>
+        <v/>
+      </c>
+      <c r="C128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
+          <t>(−) Inversión en activos fijos</t>
+        </is>
+      </c>
+      <c r="B129" s="12">
+        <f>SUM(B28:B33)</f>
+        <v/>
+      </c>
+      <c r="C129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L129" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="6" t="inlineStr">
+        <is>
+          <t>(−) Inversión en capital de trabajo</t>
+        </is>
+      </c>
+      <c r="B130" s="12">
+        <f>B85</f>
+        <v/>
+      </c>
+      <c r="C130" s="12">
+        <f>C85</f>
+        <v/>
+      </c>
+      <c r="D130" s="12">
+        <f>D85</f>
+        <v/>
+      </c>
+      <c r="E130" s="12">
+        <f>E85</f>
+        <v/>
+      </c>
+      <c r="F130" s="12">
+        <f>F85</f>
+        <v/>
+      </c>
+      <c r="G130" s="12">
+        <f>G85</f>
+        <v/>
+      </c>
+      <c r="H130" s="12">
+        <f>H85</f>
+        <v/>
+      </c>
+      <c r="I130" s="12">
+        <f>I85</f>
+        <v/>
+      </c>
+      <c r="J130" s="12">
+        <f>J85</f>
+        <v/>
+      </c>
+      <c r="K130" s="12">
+        <f>K85</f>
+        <v/>
+      </c>
+      <c r="L130" s="12">
+        <f>L85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
           <t>(−) Abono a capital del préstamo</t>
         </is>
       </c>
-      <c r="B129" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C129" s="12">
+      <c r="B131" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C131" s="12">
         <f>C91</f>
         <v/>
       </c>
-      <c r="D129" s="12">
+      <c r="D131" s="12">
         <f>D91</f>
         <v/>
       </c>
-      <c r="E129" s="12">
+      <c r="E131" s="12">
         <f>E91</f>
         <v/>
       </c>
-      <c r="F129" s="12">
+      <c r="F131" s="12">
         <f>F91</f>
         <v/>
       </c>
-      <c r="G129" s="12">
+      <c r="G131" s="12">
         <f>G91</f>
         <v/>
       </c>
-      <c r="H129" s="12">
+      <c r="H131" s="12">
         <f>H91</f>
         <v/>
       </c>
-      <c r="I129" s="12">
+      <c r="I131" s="12">
         <f>I91</f>
         <v/>
       </c>
-      <c r="J129" s="12">
+      <c r="J131" s="12">
         <f>J91</f>
         <v/>
       </c>
-      <c r="K129" s="12">
+      <c r="K131" s="12">
         <f>K91</f>
         <v/>
       </c>
-      <c r="L129" s="12">
+      <c r="L131" s="12">
         <f>L91</f>
         <v/>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="15" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="15" t="inlineStr">
         <is>
           <t>(=) FLUJO DE CAJA NETO</t>
         </is>
       </c>
-      <c r="B130" s="16">
-        <f>B122+B123+B124+B125+B126-B127-B128-B129</f>
-        <v/>
-      </c>
-      <c r="C130" s="16">
-        <f>C122+C123+C124+C125+C126-C127-C128-C129</f>
-        <v/>
-      </c>
-      <c r="D130" s="16">
-        <f>D122+D123+D124+D125+D126-D127-D128-D129</f>
-        <v/>
-      </c>
-      <c r="E130" s="16">
-        <f>E122+E123+E124+E125+E126-E127-E128-E129</f>
-        <v/>
-      </c>
-      <c r="F130" s="16">
-        <f>F122+F123+F124+F125+F126-F127-F128-F129</f>
-        <v/>
-      </c>
-      <c r="G130" s="16">
-        <f>G122+G123+G124+G125+G126-G127-G128-G129</f>
-        <v/>
-      </c>
-      <c r="H130" s="16">
-        <f>H122+H123+H124+H125+H126-H127-H128-H129</f>
-        <v/>
-      </c>
-      <c r="I130" s="16">
-        <f>I122+I123+I124+I125+I126-I127-I128-I129</f>
-        <v/>
-      </c>
-      <c r="J130" s="16">
-        <f>J122+J123+J124+J125+J126-J127-J128-J129</f>
-        <v/>
-      </c>
-      <c r="K130" s="16">
-        <f>K122+K123+K124+K125+K126-K127-K128-K129</f>
-        <v/>
-      </c>
-      <c r="L130" s="16">
-        <f>L122+L123+L124+L125+L126-L127-L128-L129</f>
-        <v/>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="21" t="inlineStr">
+      <c r="B132" s="16">
+        <f>B124+B125+B126+B127+B128-B129-B130-B131</f>
+        <v/>
+      </c>
+      <c r="C132" s="16">
+        <f>C124+C125+C126+C127+C128-C129-C130-C131</f>
+        <v/>
+      </c>
+      <c r="D132" s="16">
+        <f>D124+D125+D126+D127+D128-D129-D130-D131</f>
+        <v/>
+      </c>
+      <c r="E132" s="16">
+        <f>E124+E125+E126+E127+E128-E129-E130-E131</f>
+        <v/>
+      </c>
+      <c r="F132" s="16">
+        <f>F124+F125+F126+F127+F128-F129-F130-F131</f>
+        <v/>
+      </c>
+      <c r="G132" s="16">
+        <f>G124+G125+G126+G127+G128-G129-G130-G131</f>
+        <v/>
+      </c>
+      <c r="H132" s="16">
+        <f>H124+H125+H126+H127+H128-H129-H130-H131</f>
+        <v/>
+      </c>
+      <c r="I132" s="16">
+        <f>I124+I125+I126+I127+I128-I129-I130-I131</f>
+        <v/>
+      </c>
+      <c r="J132" s="16">
+        <f>J124+J125+J126+J127+J128-J129-J130-J131</f>
+        <v/>
+      </c>
+      <c r="K132" s="16">
+        <f>K124+K125+K126+K127+K128-K129-K130-K131</f>
+        <v/>
+      </c>
+      <c r="L132" s="16">
+        <f>L124+L125+L126+L127+L128-L129-L130-L131</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="21" t="inlineStr">
         <is>
           <t>Flujo de caja acumulado</t>
         </is>
       </c>
-      <c r="B131" s="22">
-        <f>B130</f>
-        <v/>
-      </c>
-      <c r="C131" s="22">
-        <f>B131+C130</f>
-        <v/>
-      </c>
-      <c r="D131" s="22">
-        <f>C131+D130</f>
-        <v/>
-      </c>
-      <c r="E131" s="22">
-        <f>D131+E130</f>
-        <v/>
-      </c>
-      <c r="F131" s="22">
-        <f>E131+F130</f>
-        <v/>
-      </c>
-      <c r="G131" s="22">
-        <f>F131+G130</f>
-        <v/>
-      </c>
-      <c r="H131" s="22">
-        <f>G131+H130</f>
-        <v/>
-      </c>
-      <c r="I131" s="22">
-        <f>H131+I130</f>
-        <v/>
-      </c>
-      <c r="J131" s="22">
-        <f>I131+J130</f>
-        <v/>
-      </c>
-      <c r="K131" s="22">
-        <f>J131+K130</f>
-        <v/>
-      </c>
-      <c r="L131" s="22">
-        <f>K131+L130</f>
-        <v/>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="3" t="inlineStr">
+      <c r="B133" s="22">
+        <f>B132</f>
+        <v/>
+      </c>
+      <c r="C133" s="22">
+        <f>B133+C132</f>
+        <v/>
+      </c>
+      <c r="D133" s="22">
+        <f>C133+D132</f>
+        <v/>
+      </c>
+      <c r="E133" s="22">
+        <f>D133+E132</f>
+        <v/>
+      </c>
+      <c r="F133" s="22">
+        <f>E133+F132</f>
+        <v/>
+      </c>
+      <c r="G133" s="22">
+        <f>F133+G132</f>
+        <v/>
+      </c>
+      <c r="H133" s="22">
+        <f>G133+H132</f>
+        <v/>
+      </c>
+      <c r="I133" s="22">
+        <f>H133+I132</f>
+        <v/>
+      </c>
+      <c r="J133" s="22">
+        <f>I133+J132</f>
+        <v/>
+      </c>
+      <c r="K133" s="22">
+        <f>J133+K132</f>
+        <v/>
+      </c>
+      <c r="L133" s="22">
+        <f>K133+L132</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
         <is>
           <t>11. COSTO DE CAPITAL — PROYECTO PURO (sin financiamiento)</t>
         </is>
       </c>
-      <c r="B133" s="4" t="n"/>
-      <c r="C133" s="4" t="n"/>
-      <c r="D133" s="4" t="n"/>
-      <c r="E133" s="4" t="n"/>
-      <c r="F133" s="4" t="n"/>
-      <c r="G133" s="4" t="n"/>
-      <c r="H133" s="4" t="n"/>
-      <c r="I133" s="4" t="n"/>
-      <c r="J133" s="4" t="n"/>
-      <c r="K133" s="4" t="n"/>
-      <c r="L133" s="4" t="n"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="3" t="inlineStr">
+      <c r="B135" s="4" t="n"/>
+      <c r="C135" s="4" t="n"/>
+      <c r="D135" s="4" t="n"/>
+      <c r="E135" s="4" t="n"/>
+      <c r="F135" s="4" t="n"/>
+      <c r="G135" s="4" t="n"/>
+      <c r="H135" s="4" t="n"/>
+      <c r="I135" s="4" t="n"/>
+      <c r="J135" s="4" t="n"/>
+      <c r="K135" s="4" t="n"/>
+      <c r="L135" s="4" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B134" s="5" t="inlineStr">
+      <c r="B136" s="5" t="inlineStr">
         <is>
           <t>Monto</t>
         </is>
       </c>
-      <c r="C134" s="5" t="inlineStr">
+      <c r="C136" s="5" t="inlineStr">
         <is>
           <t>Participación</t>
         </is>
       </c>
-      <c r="D134" s="5" t="inlineStr">
+      <c r="D136" s="5" t="inlineStr">
         <is>
           <t>Costo</t>
         </is>
       </c>
-      <c r="E134" s="5" t="inlineStr">
+      <c r="E136" s="5" t="inlineStr">
         <is>
           <t>Costo ponderado</t>
         </is>
       </c>
-      <c r="F134" s="4" t="n"/>
-      <c r="G134" s="4" t="n"/>
-      <c r="H134" s="4" t="n"/>
-      <c r="I134" s="4" t="n"/>
-      <c r="J134" s="4" t="n"/>
-      <c r="K134" s="4" t="n"/>
-      <c r="L134" s="4" t="n"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="6" t="inlineStr">
+      <c r="F136" s="4" t="n"/>
+      <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n"/>
+      <c r="I136" s="4" t="n"/>
+      <c r="J136" s="4" t="n"/>
+      <c r="K136" s="4" t="n"/>
+      <c r="L136" s="4" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="6" t="inlineStr">
         <is>
           <t>Recursos propios (100%)</t>
         </is>
       </c>
-      <c r="B135" s="12">
+      <c r="B137" s="12">
         <f>B35</f>
         <v/>
       </c>
-      <c r="C135" s="23">
-        <f>B135/B136</f>
-        <v/>
-      </c>
-      <c r="D135" s="23">
+      <c r="C137" s="23">
+        <f>B137/B138</f>
+        <v/>
+      </c>
+      <c r="D137" s="23">
         <f>$B$12</f>
         <v/>
       </c>
-      <c r="E135" s="23">
-        <f>C135*D135</f>
-        <v/>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="15" t="inlineStr">
+      <c r="E137" s="23">
+        <f>C137*D137</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="15" t="inlineStr">
         <is>
           <t>TOTAL / Tasa de descuento del proyecto</t>
         </is>
       </c>
-      <c r="B136" s="16">
-        <f>B135</f>
-        <v/>
-      </c>
-      <c r="C136" s="24" t="n">
+      <c r="B138" s="16">
+        <f>B137</f>
+        <v/>
+      </c>
+      <c r="C138" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D136" s="25" t="inlineStr">
+      <c r="D138" s="25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E136" s="24">
-        <f>E135</f>
-        <v/>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="3" t="inlineStr">
+      <c r="E138" s="24">
+        <f>E137</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
         <is>
           <t>12. INDICADORES FINANCIEROS — PROYECTO PURO</t>
         </is>
       </c>
-      <c r="B138" s="4" t="n"/>
-      <c r="C138" s="4" t="n"/>
-      <c r="D138" s="4" t="n"/>
-      <c r="E138" s="4" t="n"/>
-      <c r="F138" s="4" t="n"/>
-      <c r="G138" s="4" t="n"/>
-      <c r="H138" s="4" t="n"/>
-      <c r="I138" s="4" t="n"/>
-      <c r="J138" s="4" t="n"/>
-      <c r="K138" s="4" t="n"/>
-      <c r="L138" s="4" t="n"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="21" t="inlineStr">
-        <is>
-          <t>VAN (Valor Actual Neto)</t>
-        </is>
-      </c>
-      <c r="B139" s="8">
-        <f>NPV(E136,C110:L110)+B110</f>
-        <v/>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="21" t="inlineStr">
-        <is>
-          <t>TIR (Tasa Interna de Retorno)</t>
-        </is>
-      </c>
-      <c r="B140" s="7">
-        <f>IRR(B110:L110)</f>
-        <v/>
-      </c>
+      <c r="B140" s="4" t="n"/>
+      <c r="C140" s="4" t="n"/>
+      <c r="D140" s="4" t="n"/>
+      <c r="E140" s="4" t="n"/>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n"/>
+      <c r="I140" s="4" t="n"/>
+      <c r="J140" s="4" t="n"/>
+      <c r="K140" s="4" t="n"/>
+      <c r="L140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="21" t="inlineStr">
         <is>
-          <t>PRI (años de recuperación)</t>
-        </is>
-      </c>
-      <c r="B141" s="9">
-        <f>IF(COUNTIF(B111:L111,"&lt;0")=11,"&gt;10",(COUNTIF(B111:L111,"&lt;0")-1)+(-INDEX(B111:L111,COUNTIF(B111:L111,"&lt;0")))/INDEX(B110:L110,COUNTIF(B111:L111,"&lt;0")+1))</f>
+          <t>VAN (Valor Actual Neto)</t>
+        </is>
+      </c>
+      <c r="B141" s="8">
+        <f>NPV(E138,C111:L111)+B111</f>
         <v/>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="21" t="inlineStr">
         <is>
+          <t>TIR (Tasa Interna de Retorno)</t>
+        </is>
+      </c>
+      <c r="B142" s="7">
+        <f>IRR(B111:L111)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="21" t="inlineStr">
+        <is>
+          <t>PRI (años de recuperación)</t>
+        </is>
+      </c>
+      <c r="B143" s="9">
+        <f>IF(COUNTIF(B112:L112,"&lt;0")=11,"&gt;10",(COUNTIF(B112:L112,"&lt;0")-1)+(-INDEX(B112:L112,COUNTIF(B112:L112,"&lt;0")))/INDEX(B111:L111,COUNTIF(B112:L112,"&lt;0")+1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="21" t="inlineStr">
+        <is>
           <t>Relación Beneficio/Costo</t>
         </is>
       </c>
-      <c r="B142" s="9">
-        <f>NPV(E136,C42:L42)/(B35+NPV(E136,C49:L49)+NPV(E136,C69:L69)+NPV(E136,C103:L103))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="3" t="inlineStr">
+      <c r="B144" s="9">
+        <f>NPV(E138,C42:L42)/(B35+NPV(E138,C49:L49)+NPV(E138,C69:L69)+NPV(E138,C104:L104))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
         <is>
           <t>13. COSTO DE CAPITAL — CON FINANCIAMIENTO (WACC)</t>
         </is>
       </c>
-      <c r="B144" s="4" t="n"/>
-      <c r="C144" s="4" t="n"/>
-      <c r="D144" s="4" t="n"/>
-      <c r="E144" s="4" t="n"/>
-      <c r="F144" s="4" t="n"/>
-      <c r="G144" s="4" t="n"/>
-      <c r="H144" s="4" t="n"/>
-      <c r="I144" s="4" t="n"/>
-      <c r="J144" s="4" t="n"/>
-      <c r="K144" s="4" t="n"/>
-      <c r="L144" s="4" t="n"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="3" t="inlineStr">
+      <c r="B146" s="4" t="n"/>
+      <c r="C146" s="4" t="n"/>
+      <c r="D146" s="4" t="n"/>
+      <c r="E146" s="4" t="n"/>
+      <c r="F146" s="4" t="n"/>
+      <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n"/>
+      <c r="I146" s="4" t="n"/>
+      <c r="J146" s="4" t="n"/>
+      <c r="K146" s="4" t="n"/>
+      <c r="L146" s="4" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="B145" s="5" t="inlineStr">
+      <c r="B147" s="5" t="inlineStr">
         <is>
           <t>Monto</t>
         </is>
       </c>
-      <c r="C145" s="5" t="inlineStr">
+      <c r="C147" s="5" t="inlineStr">
         <is>
           <t>Participación</t>
         </is>
       </c>
-      <c r="D145" s="5" t="inlineStr">
+      <c r="D147" s="5" t="inlineStr">
         <is>
           <t>Costo</t>
         </is>
       </c>
-      <c r="E145" s="5" t="inlineStr">
+      <c r="E147" s="5" t="inlineStr">
         <is>
           <t>Costo ponderado</t>
         </is>
       </c>
-      <c r="F145" s="4" t="n"/>
-      <c r="G145" s="4" t="n"/>
-      <c r="H145" s="4" t="n"/>
-      <c r="I145" s="4" t="n"/>
-      <c r="J145" s="4" t="n"/>
-      <c r="K145" s="4" t="n"/>
-      <c r="L145" s="4" t="n"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="6" t="inlineStr">
+      <c r="F147" s="4" t="n"/>
+      <c r="G147" s="4" t="n"/>
+      <c r="H147" s="4" t="n"/>
+      <c r="I147" s="4" t="n"/>
+      <c r="J147" s="4" t="n"/>
+      <c r="K147" s="4" t="n"/>
+      <c r="L147" s="4" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="6" t="inlineStr">
         <is>
           <t>Préstamo bancario (deuda, después de impuestos)</t>
         </is>
       </c>
-      <c r="B146" s="12">
+      <c r="B148" s="12">
         <f>D35</f>
         <v/>
       </c>
-      <c r="C146" s="23">
-        <f>B146/B148</f>
-        <v/>
-      </c>
-      <c r="D146" s="23">
+      <c r="C148" s="23">
+        <f>B148/B150</f>
+        <v/>
+      </c>
+      <c r="D148" s="23">
         <f>$B$9*(1-$B$6)</f>
         <v/>
       </c>
-      <c r="E146" s="23">
-        <f>C146*D146</f>
-        <v/>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="6" t="inlineStr">
+      <c r="E148" s="23">
+        <f>C148*D148</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="6" t="inlineStr">
         <is>
           <t>Recursos propios (patrimonio)</t>
         </is>
       </c>
-      <c r="B147" s="12">
+      <c r="B149" s="12">
         <f>C35</f>
         <v/>
       </c>
-      <c r="C147" s="23">
-        <f>B147/B148</f>
-        <v/>
-      </c>
-      <c r="D147" s="23">
+      <c r="C149" s="23">
+        <f>B149/B150</f>
+        <v/>
+      </c>
+      <c r="D149" s="23">
         <f>$B$12</f>
         <v/>
       </c>
-      <c r="E147" s="23">
-        <f>C147*D147</f>
-        <v/>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="15" t="inlineStr">
+      <c r="E149" s="23">
+        <f>C149*D149</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="15" t="inlineStr">
         <is>
           <t>TOTAL / WACC</t>
         </is>
       </c>
-      <c r="B148" s="16">
-        <f>B146+B147</f>
-        <v/>
-      </c>
-      <c r="C148" s="24" t="n">
+      <c r="B150" s="16">
+        <f>B148+B149</f>
+        <v/>
+      </c>
+      <c r="C150" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="D148" s="25" t="inlineStr">
+      <c r="D150" s="25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E148" s="24">
-        <f>E146+E147</f>
-        <v/>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="3" t="inlineStr">
+      <c r="E150" s="24">
+        <f>E148+E149</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
         <is>
           <t>14. INDICADORES FINANCIEROS — CON FINANCIAMIENTO</t>
         </is>
       </c>
-      <c r="B150" s="4" t="n"/>
-      <c r="C150" s="4" t="n"/>
-      <c r="D150" s="4" t="n"/>
-      <c r="E150" s="4" t="n"/>
-      <c r="F150" s="4" t="n"/>
-      <c r="G150" s="4" t="n"/>
-      <c r="H150" s="4" t="n"/>
-      <c r="I150" s="4" t="n"/>
-      <c r="J150" s="4" t="n"/>
-      <c r="K150" s="4" t="n"/>
-      <c r="L150" s="4" t="n"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="21" t="inlineStr">
-        <is>
-          <t>VAN (Valor Actual Neto)</t>
-        </is>
-      </c>
-      <c r="B151" s="8">
-        <f>NPV(E148,C130:L130)+B130</f>
-        <v/>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="21" t="inlineStr">
-        <is>
-          <t>TIR (Tasa Interna de Retorno)</t>
-        </is>
-      </c>
-      <c r="B152" s="7">
-        <f>IRR(B130:L130)</f>
-        <v/>
-      </c>
+      <c r="B152" s="4" t="n"/>
+      <c r="C152" s="4" t="n"/>
+      <c r="D152" s="4" t="n"/>
+      <c r="E152" s="4" t="n"/>
+      <c r="F152" s="4" t="n"/>
+      <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="n"/>
+      <c r="I152" s="4" t="n"/>
+      <c r="J152" s="4" t="n"/>
+      <c r="K152" s="4" t="n"/>
+      <c r="L152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="21" t="inlineStr">
         <is>
-          <t>PRI (años de recuperación)</t>
-        </is>
-      </c>
-      <c r="B153" s="9">
-        <f>IF(COUNTIF(B131:L131,"&lt;0")=11,"&gt;10",(COUNTIF(B131:L131,"&lt;0")-1)+(-INDEX(B131:L131,COUNTIF(B131:L131,"&lt;0")))/INDEX(B130:L130,COUNTIF(B131:L131,"&lt;0")+1))</f>
+          <t>VAN (Valor Actual Neto)</t>
+        </is>
+      </c>
+      <c r="B153" s="8">
+        <f>NPV(E150,C132:L132)+B132</f>
         <v/>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="21" t="inlineStr">
         <is>
+          <t>TIR (Tasa Interna de Retorno)</t>
+        </is>
+      </c>
+      <c r="B154" s="7">
+        <f>IRR(B132:L132)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="21" t="inlineStr">
+        <is>
+          <t>PRI (años de recuperación)</t>
+        </is>
+      </c>
+      <c r="B155" s="9">
+        <f>IF(COUNTIF(B133:L133,"&lt;0")=11,"&gt;10",(COUNTIF(B133:L133,"&lt;0")-1)+(-INDEX(B133:L133,COUNTIF(B133:L133,"&lt;0")))/INDEX(B132:L132,COUNTIF(B133:L133,"&lt;0")+1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="21" t="inlineStr">
+        <is>
           <t>Relación Beneficio/Costo</t>
         </is>
       </c>
-      <c r="B154" s="9">
-        <f>NPV(E148,C42:L42)/(C35+NPV(E148,C49:L49)+NPV(E148,C69:L69)+NPV(E148,C118:L118)+NPV(E148,C121:L121)+NPV(E148,C129:L129))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="3" t="inlineStr">
+      <c r="B156" s="9">
+        <f>NPV(E150,C42:L42)/(C35+NPV(E150,C49:L49)+NPV(E150,C69:L69)+NPV(E150,C119:L119)+NPV(E150,C123:L123)+NPV(E150,C131:L131))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
         <is>
           <t>15. NOTAS LEGALES (cumplimiento normativo Honduras)</t>
         </is>
       </c>
-      <c r="B156" s="4" t="n"/>
-      <c r="C156" s="4" t="n"/>
-      <c r="D156" s="4" t="n"/>
-      <c r="E156" s="4" t="n"/>
-      <c r="F156" s="4" t="n"/>
-      <c r="G156" s="4" t="n"/>
-      <c r="H156" s="4" t="n"/>
-      <c r="I156" s="4" t="n"/>
-      <c r="J156" s="4" t="n"/>
-      <c r="K156" s="4" t="n"/>
-      <c r="L156" s="4" t="n"/>
-    </row>
-    <row r="157" ht="30" customHeight="1">
-      <c r="A157" s="26" t="inlineStr">
-        <is>
-          <t>• ISR: 25% + aportación solidaria 5% sobre el excedente de L 1,000,000 (Ley del ISR).</t>
-        </is>
-      </c>
-      <c r="B157" s="14" t="n"/>
-      <c r="C157" s="14" t="n"/>
-      <c r="D157" s="14" t="n"/>
-      <c r="E157" s="14" t="n"/>
-      <c r="F157" s="14" t="n"/>
-      <c r="G157" s="14" t="n"/>
-      <c r="H157" s="14" t="n"/>
-      <c r="I157" s="14" t="n"/>
-      <c r="J157" s="14" t="n"/>
-      <c r="K157" s="14" t="n"/>
-      <c r="L157" s="14" t="n"/>
-    </row>
-    <row r="158" ht="30" customHeight="1">
-      <c r="A158" s="26" t="inlineStr">
-        <is>
-          <t>• Depreciación línea recta: maquinaria 10%; vehículos 10%-33% (aquí 20% = 5 años); diferidos 5 años.</t>
-        </is>
-      </c>
-      <c r="B158" s="14" t="n"/>
-      <c r="C158" s="14" t="n"/>
-      <c r="D158" s="14" t="n"/>
-      <c r="E158" s="14" t="n"/>
-      <c r="F158" s="14" t="n"/>
-      <c r="G158" s="14" t="n"/>
-      <c r="H158" s="14" t="n"/>
-      <c r="I158" s="14" t="n"/>
-      <c r="J158" s="14" t="n"/>
-      <c r="K158" s="14" t="n"/>
-      <c r="L158" s="14" t="n"/>
+      <c r="B158" s="4" t="n"/>
+      <c r="C158" s="4" t="n"/>
+      <c r="D158" s="4" t="n"/>
+      <c r="E158" s="4" t="n"/>
+      <c r="F158" s="4" t="n"/>
+      <c r="G158" s="4" t="n"/>
+      <c r="H158" s="4" t="n"/>
+      <c r="I158" s="4" t="n"/>
+      <c r="J158" s="4" t="n"/>
+      <c r="K158" s="4" t="n"/>
+      <c r="L158" s="4" t="n"/>
     </row>
     <row r="159" ht="30" customHeight="1">
       <c r="A159" s="26" t="inlineStr">
         <is>
-          <t>• Seguridad social patronal (techo L 11,903.13): IHSS EM 2.5% + IVM 1% + RP 0.2% + RAP 1.5%; INFOP 1% sobre planilla (sin techo).</t>
+          <t>• ISR: 25% + aportación solidaria 5% sobre el excedente de L 1,000,000 (Ley del ISR).</t>
         </is>
       </c>
       <c r="B159" s="14" t="n"/>
@@ -5364,7 +5426,7 @@
     <row r="160" ht="30" customHeight="1">
       <c r="A160" s="26" t="inlineStr">
         <is>
-          <t>• Prestaciones: aguinaldo (13.º mes) y catorceavo (14.º mes) — Código del Trabajo.</t>
+          <t>• Depreciación línea recta: maquinaria 10%; vehículos 10%-33% (aquí 20% = 5 años); diferidos 5 años.</t>
         </is>
       </c>
       <c r="B160" s="14" t="n"/>
@@ -5382,7 +5444,7 @@
     <row r="161" ht="30" customHeight="1">
       <c r="A161" s="26" t="inlineStr">
         <is>
-          <t>• ISV: la leche fluida/pasteurizada está exenta; no se cobra ISV en ventas.</t>
+          <t>• Seguridad social patronal (techo L 11,903.13): IHSS EM 2.5% + IVM 1% + RP 0.2% + RAP 1.5%; INFOP 1% sobre planilla (sin techo).</t>
         </is>
       </c>
       <c r="B161" s="14" t="n"/>
@@ -5400,7 +5462,7 @@
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="26" t="inlineStr">
         <is>
-          <t>• Impuesto al Activo Neto 1% (deducción L3M; exento en preoperación; se paga solo si supera al ISR).</t>
+          <t>• Prestaciones: aguinaldo (13.º mes) y catorceavo (14.º mes) — Código del Trabajo.</t>
         </is>
       </c>
       <c r="B162" s="14" t="n"/>
@@ -5418,7 +5480,7 @@
     <row r="163" ht="30" customHeight="1">
       <c r="A163" s="26" t="inlineStr">
         <is>
-          <t>• Manufactura puede arrastrar pérdidas fiscales 3 años (no aplicado, criterio conservador).</t>
+          <t>• ISV: la leche fluida/pasteurizada está exenta; no se cobra ISV en ventas.</t>
         </is>
       </c>
       <c r="B163" s="14" t="n"/>
@@ -5436,7 +5498,7 @@
     <row r="164" ht="30" customHeight="1">
       <c r="A164" s="26" t="inlineStr">
         <is>
-          <t>• Impuestos municipales de Comayagua (industria, comercio y servicios; bienes inmuebles).</t>
+          <t>• Arrastre de pérdidas fiscales: la manufactura puede compensarlas hasta 3 años (aplicado en el flujo, línea de pérdidas acumuladas).</t>
         </is>
       </c>
       <c r="B164" s="14" t="n"/>
@@ -5451,38 +5513,93 @@
       <c r="K164" s="14" t="n"/>
       <c r="L164" s="14" t="n"/>
     </row>
+    <row r="165" ht="30" customHeight="1">
+      <c r="A165" s="26" t="inlineStr">
+        <is>
+          <t>• Impuesto al Activo Neto 1% (deducción L3M; exento en preoperación; se paga solo si supera al ISR).</t>
+        </is>
+      </c>
+      <c r="B165" s="14" t="n"/>
+      <c r="C165" s="14" t="n"/>
+      <c r="D165" s="14" t="n"/>
+      <c r="E165" s="14" t="n"/>
+      <c r="F165" s="14" t="n"/>
+      <c r="G165" s="14" t="n"/>
+      <c r="H165" s="14" t="n"/>
+      <c r="I165" s="14" t="n"/>
+      <c r="J165" s="14" t="n"/>
+      <c r="K165" s="14" t="n"/>
+      <c r="L165" s="14" t="n"/>
+    </row>
+    <row r="166" ht="30" customHeight="1">
+      <c r="A166" s="26" t="inlineStr">
+        <is>
+          <t>• Capital de trabajo: 1 mes de costos operativos, financiado con crédito de proveedores (CREL/ganaderos).</t>
+        </is>
+      </c>
+      <c r="B166" s="14" t="n"/>
+      <c r="C166" s="14" t="n"/>
+      <c r="D166" s="14" t="n"/>
+      <c r="E166" s="14" t="n"/>
+      <c r="F166" s="14" t="n"/>
+      <c r="G166" s="14" t="n"/>
+      <c r="H166" s="14" t="n"/>
+      <c r="I166" s="14" t="n"/>
+      <c r="J166" s="14" t="n"/>
+      <c r="K166" s="14" t="n"/>
+      <c r="L166" s="14" t="n"/>
+    </row>
+    <row r="167" ht="30" customHeight="1">
+      <c r="A167" s="26" t="inlineStr">
+        <is>
+          <t>• Impuestos municipales de Comayagua (industria, comercio y servicios; bienes inmuebles).</t>
+        </is>
+      </c>
+      <c r="B167" s="14" t="n"/>
+      <c r="C167" s="14" t="n"/>
+      <c r="D167" s="14" t="n"/>
+      <c r="E167" s="14" t="n"/>
+      <c r="F167" s="14" t="n"/>
+      <c r="G167" s="14" t="n"/>
+      <c r="H167" s="14" t="n"/>
+      <c r="I167" s="14" t="n"/>
+      <c r="J167" s="14" t="n"/>
+      <c r="K167" s="14" t="n"/>
+      <c r="L167" s="14" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="D57:L57"/>
     <mergeCell ref="A164:L164"/>
     <mergeCell ref="A37:L37"/>
-    <mergeCell ref="A133:L133"/>
     <mergeCell ref="A158:L158"/>
     <mergeCell ref="D53:L53"/>
     <mergeCell ref="A163:L163"/>
     <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A113:L113"/>
     <mergeCell ref="A71:L71"/>
     <mergeCell ref="A160:L160"/>
     <mergeCell ref="D56:L56"/>
     <mergeCell ref="D58:L58"/>
     <mergeCell ref="A159:L159"/>
-    <mergeCell ref="A150:L150"/>
-    <mergeCell ref="A144:L144"/>
+    <mergeCell ref="A135:L135"/>
+    <mergeCell ref="A140:L140"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="D55:L55"/>
     <mergeCell ref="A81:L81"/>
     <mergeCell ref="A96:L96"/>
-    <mergeCell ref="A156:L156"/>
+    <mergeCell ref="A165:L165"/>
     <mergeCell ref="A161:L161"/>
+    <mergeCell ref="A152:L152"/>
     <mergeCell ref="D54:L54"/>
     <mergeCell ref="A44:L44"/>
+    <mergeCell ref="A167:L167"/>
     <mergeCell ref="D59:L59"/>
-    <mergeCell ref="A157:L157"/>
+    <mergeCell ref="A114:L114"/>
     <mergeCell ref="A64:L64"/>
+    <mergeCell ref="A166:L166"/>
     <mergeCell ref="A51:L51"/>
-    <mergeCell ref="A138:L138"/>
     <mergeCell ref="A88:L88"/>
+    <mergeCell ref="A146:L146"/>
     <mergeCell ref="A162:L162"/>
     <mergeCell ref="C60:L60"/>
     <mergeCell ref="D52:L52"/>
@@ -5497,7 +5614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5711,7 +5828,7 @@
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>Incluir 2 meses de costos, recuperar Año 10</t>
+          <t>1 mes de costos (crédito proveedores), recuperado Año 10</t>
         </is>
       </c>
     </row>
@@ -5721,17 +5838,17 @@
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>Estudio de personal</t>
+          <t>Estudio financiero</t>
         </is>
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>Faltan cargas sociales de ley</t>
+          <t>No aprovecha arrastre de pérdidas</t>
         </is>
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>IHSS+RAP (con techo)+INFOP+aguinaldo+catorceavo</t>
+          <t>Compensar pérdidas de años iniciales (ley, 3 años)</t>
         </is>
       </c>
     </row>
@@ -5741,17 +5858,37 @@
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
+          <t>Estudio de personal</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="inlineStr">
+        <is>
+          <t>Faltan cargas sociales de ley</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>IHSS+RAP (con techo)+INFOP+aguinaldo+catorceavo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
           <t>Cuadro 1 / ventas</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>Captación lenta (15 clientes) y consumo bajo (60 L/mes)</t>
-        </is>
-      </c>
-      <c r="D13" s="26" t="inlineStr">
-        <is>
-          <t>Captación agresiva (60→690 clientes) y consumo realista 150 L/mes</t>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t>Captación lenta (15 clientes)</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Captación agresiva (60→690 clientes), consumo 150 L/mes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reemplaza TIR por TIRM (MIRR) ajustada: reinversion al costo de capital (proyecto 37.18%, financiamiento 38.97%); Excel y tesis congruentes
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -56,7 +56,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -78,11 +78,55 @@
         <color rgb="FFBFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -150,6 +194,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -552,17 +598,17 @@
           <t>SUPUESTOS BASE DEL PROYECTO</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="27" t="n"/>
+      <c r="E4" s="27" t="n"/>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+      <c r="H4" s="27" t="n"/>
+      <c r="I4" s="27" t="n"/>
+      <c r="J4" s="27" t="n"/>
+      <c r="K4" s="27" t="n"/>
+      <c r="L4" s="28" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -774,17 +820,17 @@
           <t>1. PLAN DE INVERSIONES Y FINANCIAMIENTO</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
+      <c r="B26" s="27" t="n"/>
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="27" t="n"/>
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="27" t="n"/>
+      <c r="H26" s="27" t="n"/>
+      <c r="I26" s="27" t="n"/>
+      <c r="J26" s="27" t="n"/>
+      <c r="K26" s="27" t="n"/>
+      <c r="L26" s="28" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1084,17 +1130,17 @@
           <t>2. PRODUCCIÓN Y VENTAS  (volumen = clientes × consumo mensual × 12)</t>
         </is>
       </c>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-      <c r="D37" s="4" t="n"/>
-      <c r="E37" s="4" t="n"/>
-      <c r="F37" s="4" t="n"/>
-      <c r="G37" s="4" t="n"/>
-      <c r="H37" s="4" t="n"/>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
-      <c r="L37" s="4" t="n"/>
+      <c r="B37" s="27" t="n"/>
+      <c r="C37" s="27" t="n"/>
+      <c r="D37" s="27" t="n"/>
+      <c r="E37" s="27" t="n"/>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
+      <c r="H37" s="27" t="n"/>
+      <c r="I37" s="27" t="n"/>
+      <c r="J37" s="27" t="n"/>
+      <c r="K37" s="27" t="n"/>
+      <c r="L37" s="28" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1345,17 +1391,17 @@
           <t>3. COSTOS VARIABLES  (= litros × costo unitario × inflación)</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-      <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="n"/>
-      <c r="J44" s="4" t="n"/>
-      <c r="K44" s="4" t="n"/>
-      <c r="L44" s="4" t="n"/>
+      <c r="B44" s="27" t="n"/>
+      <c r="C44" s="27" t="n"/>
+      <c r="D44" s="27" t="n"/>
+      <c r="E44" s="27" t="n"/>
+      <c r="F44" s="27" t="n"/>
+      <c r="G44" s="27" t="n"/>
+      <c r="H44" s="27" t="n"/>
+      <c r="I44" s="27" t="n"/>
+      <c r="J44" s="27" t="n"/>
+      <c r="K44" s="27" t="n"/>
+      <c r="L44" s="28" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -1626,17 +1672,17 @@
           <t>4. COSTO DE PERSONAL  (con prestaciones y seguridad social de ley)</t>
         </is>
       </c>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
-      <c r="K51" s="4" t="n"/>
-      <c r="L51" s="4" t="n"/>
+      <c r="B51" s="27" t="n"/>
+      <c r="C51" s="27" t="n"/>
+      <c r="D51" s="27" t="n"/>
+      <c r="E51" s="27" t="n"/>
+      <c r="F51" s="27" t="n"/>
+      <c r="G51" s="27" t="n"/>
+      <c r="H51" s="27" t="n"/>
+      <c r="I51" s="27" t="n"/>
+      <c r="J51" s="27" t="n"/>
+      <c r="K51" s="27" t="n"/>
+      <c r="L51" s="28" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -1655,14 +1701,14 @@
         </is>
       </c>
       <c r="D52" s="18" t="inlineStr"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-      <c r="H52" s="4" t="n"/>
-      <c r="I52" s="4" t="n"/>
-      <c r="J52" s="4" t="n"/>
-      <c r="K52" s="4" t="n"/>
-      <c r="L52" s="4" t="n"/>
+      <c r="E52" s="27" t="n"/>
+      <c r="F52" s="27" t="n"/>
+      <c r="G52" s="27" t="n"/>
+      <c r="H52" s="27" t="n"/>
+      <c r="I52" s="27" t="n"/>
+      <c r="J52" s="27" t="n"/>
+      <c r="K52" s="27" t="n"/>
+      <c r="L52" s="28" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -1678,14 +1724,14 @@
         <v/>
       </c>
       <c r="D53" s="19" t="inlineStr"/>
-      <c r="E53" s="14" t="n"/>
-      <c r="F53" s="14" t="n"/>
-      <c r="G53" s="14" t="n"/>
-      <c r="H53" s="14" t="n"/>
-      <c r="I53" s="14" t="n"/>
-      <c r="J53" s="14" t="n"/>
-      <c r="K53" s="14" t="n"/>
-      <c r="L53" s="14" t="n"/>
+      <c r="E53" s="27" t="n"/>
+      <c r="F53" s="27" t="n"/>
+      <c r="G53" s="27" t="n"/>
+      <c r="H53" s="27" t="n"/>
+      <c r="I53" s="27" t="n"/>
+      <c r="J53" s="27" t="n"/>
+      <c r="K53" s="27" t="n"/>
+      <c r="L53" s="28" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -1701,14 +1747,14 @@
         <v/>
       </c>
       <c r="D54" s="19" t="inlineStr"/>
-      <c r="E54" s="14" t="n"/>
-      <c r="F54" s="14" t="n"/>
-      <c r="G54" s="14" t="n"/>
-      <c r="H54" s="14" t="n"/>
-      <c r="I54" s="14" t="n"/>
-      <c r="J54" s="14" t="n"/>
-      <c r="K54" s="14" t="n"/>
-      <c r="L54" s="14" t="n"/>
+      <c r="E54" s="27" t="n"/>
+      <c r="F54" s="27" t="n"/>
+      <c r="G54" s="27" t="n"/>
+      <c r="H54" s="27" t="n"/>
+      <c r="I54" s="27" t="n"/>
+      <c r="J54" s="27" t="n"/>
+      <c r="K54" s="27" t="n"/>
+      <c r="L54" s="28" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -1724,14 +1770,14 @@
         <v/>
       </c>
       <c r="D55" s="19" t="inlineStr"/>
-      <c r="E55" s="14" t="n"/>
-      <c r="F55" s="14" t="n"/>
-      <c r="G55" s="14" t="n"/>
-      <c r="H55" s="14" t="n"/>
-      <c r="I55" s="14" t="n"/>
-      <c r="J55" s="14" t="n"/>
-      <c r="K55" s="14" t="n"/>
-      <c r="L55" s="14" t="n"/>
+      <c r="E55" s="27" t="n"/>
+      <c r="F55" s="27" t="n"/>
+      <c r="G55" s="27" t="n"/>
+      <c r="H55" s="27" t="n"/>
+      <c r="I55" s="27" t="n"/>
+      <c r="J55" s="27" t="n"/>
+      <c r="K55" s="27" t="n"/>
+      <c r="L55" s="28" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -1747,14 +1793,14 @@
         <v/>
       </c>
       <c r="D56" s="19" t="inlineStr"/>
-      <c r="E56" s="14" t="n"/>
-      <c r="F56" s="14" t="n"/>
-      <c r="G56" s="14" t="n"/>
-      <c r="H56" s="14" t="n"/>
-      <c r="I56" s="14" t="n"/>
-      <c r="J56" s="14" t="n"/>
-      <c r="K56" s="14" t="n"/>
-      <c r="L56" s="14" t="n"/>
+      <c r="E56" s="27" t="n"/>
+      <c r="F56" s="27" t="n"/>
+      <c r="G56" s="27" t="n"/>
+      <c r="H56" s="27" t="n"/>
+      <c r="I56" s="27" t="n"/>
+      <c r="J56" s="27" t="n"/>
+      <c r="K56" s="27" t="n"/>
+      <c r="L56" s="28" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -1770,14 +1816,14 @@
         <v/>
       </c>
       <c r="D57" s="19" t="inlineStr"/>
-      <c r="E57" s="14" t="n"/>
-      <c r="F57" s="14" t="n"/>
-      <c r="G57" s="14" t="n"/>
-      <c r="H57" s="14" t="n"/>
-      <c r="I57" s="14" t="n"/>
-      <c r="J57" s="14" t="n"/>
-      <c r="K57" s="14" t="n"/>
-      <c r="L57" s="14" t="n"/>
+      <c r="E57" s="27" t="n"/>
+      <c r="F57" s="27" t="n"/>
+      <c r="G57" s="27" t="n"/>
+      <c r="H57" s="27" t="n"/>
+      <c r="I57" s="27" t="n"/>
+      <c r="J57" s="27" t="n"/>
+      <c r="K57" s="27" t="n"/>
+      <c r="L57" s="28" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -1793,14 +1839,14 @@
         <v/>
       </c>
       <c r="D58" s="19" t="inlineStr"/>
-      <c r="E58" s="14" t="n"/>
-      <c r="F58" s="14" t="n"/>
-      <c r="G58" s="14" t="n"/>
-      <c r="H58" s="14" t="n"/>
-      <c r="I58" s="14" t="n"/>
-      <c r="J58" s="14" t="n"/>
-      <c r="K58" s="14" t="n"/>
-      <c r="L58" s="14" t="n"/>
+      <c r="E58" s="27" t="n"/>
+      <c r="F58" s="27" t="n"/>
+      <c r="G58" s="27" t="n"/>
+      <c r="H58" s="27" t="n"/>
+      <c r="I58" s="27" t="n"/>
+      <c r="J58" s="27" t="n"/>
+      <c r="K58" s="27" t="n"/>
+      <c r="L58" s="28" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
@@ -1817,14 +1863,14 @@
         <v/>
       </c>
       <c r="D59" s="20" t="inlineStr"/>
-      <c r="E59" s="17" t="n"/>
-      <c r="F59" s="17" t="n"/>
-      <c r="G59" s="17" t="n"/>
-      <c r="H59" s="17" t="n"/>
-      <c r="I59" s="17" t="n"/>
-      <c r="J59" s="17" t="n"/>
-      <c r="K59" s="17" t="n"/>
-      <c r="L59" s="17" t="n"/>
+      <c r="E59" s="27" t="n"/>
+      <c r="F59" s="27" t="n"/>
+      <c r="G59" s="27" t="n"/>
+      <c r="H59" s="27" t="n"/>
+      <c r="I59" s="27" t="n"/>
+      <c r="J59" s="27" t="n"/>
+      <c r="K59" s="27" t="n"/>
+      <c r="L59" s="28" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -1837,15 +1883,15 @@
         <v/>
       </c>
       <c r="C60" s="19" t="inlineStr"/>
-      <c r="D60" s="14" t="n"/>
-      <c r="E60" s="14" t="n"/>
-      <c r="F60" s="14" t="n"/>
-      <c r="G60" s="14" t="n"/>
-      <c r="H60" s="14" t="n"/>
-      <c r="I60" s="14" t="n"/>
-      <c r="J60" s="14" t="n"/>
-      <c r="K60" s="14" t="n"/>
-      <c r="L60" s="14" t="n"/>
+      <c r="D60" s="27" t="n"/>
+      <c r="E60" s="27" t="n"/>
+      <c r="F60" s="27" t="n"/>
+      <c r="G60" s="27" t="n"/>
+      <c r="H60" s="27" t="n"/>
+      <c r="I60" s="27" t="n"/>
+      <c r="J60" s="27" t="n"/>
+      <c r="K60" s="27" t="n"/>
+      <c r="L60" s="28" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -1965,17 +2011,17 @@
           <t>5. COSTOS FIJOS (anuales)</t>
         </is>
       </c>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-      <c r="D64" s="4" t="n"/>
-      <c r="E64" s="4" t="n"/>
-      <c r="F64" s="4" t="n"/>
-      <c r="G64" s="4" t="n"/>
-      <c r="H64" s="4" t="n"/>
-      <c r="I64" s="4" t="n"/>
-      <c r="J64" s="4" t="n"/>
-      <c r="K64" s="4" t="n"/>
-      <c r="L64" s="4" t="n"/>
+      <c r="B64" s="27" t="n"/>
+      <c r="C64" s="27" t="n"/>
+      <c r="D64" s="27" t="n"/>
+      <c r="E64" s="27" t="n"/>
+      <c r="F64" s="27" t="n"/>
+      <c r="G64" s="27" t="n"/>
+      <c r="H64" s="27" t="n"/>
+      <c r="I64" s="27" t="n"/>
+      <c r="J64" s="27" t="n"/>
+      <c r="K64" s="27" t="n"/>
+      <c r="L64" s="28" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -2247,17 +2293,17 @@
           <t>6. DEPRECIACIONES Y AMORTIZACIONES  (línea recta = Valor ÷ Vida)</t>
         </is>
       </c>
-      <c r="B71" s="4" t="n"/>
-      <c r="C71" s="4" t="n"/>
-      <c r="D71" s="4" t="n"/>
-      <c r="E71" s="4" t="n"/>
-      <c r="F71" s="4" t="n"/>
-      <c r="G71" s="4" t="n"/>
-      <c r="H71" s="4" t="n"/>
-      <c r="I71" s="4" t="n"/>
-      <c r="J71" s="4" t="n"/>
-      <c r="K71" s="4" t="n"/>
-      <c r="L71" s="4" t="n"/>
+      <c r="B71" s="27" t="n"/>
+      <c r="C71" s="27" t="n"/>
+      <c r="D71" s="27" t="n"/>
+      <c r="E71" s="27" t="n"/>
+      <c r="F71" s="27" t="n"/>
+      <c r="G71" s="27" t="n"/>
+      <c r="H71" s="27" t="n"/>
+      <c r="I71" s="27" t="n"/>
+      <c r="J71" s="27" t="n"/>
+      <c r="K71" s="27" t="n"/>
+      <c r="L71" s="28" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -2674,17 +2720,17 @@
           <t>7. VALOR DE DESECHO Y CAPITAL DE TRABAJO</t>
         </is>
       </c>
-      <c r="B81" s="4" t="n"/>
-      <c r="C81" s="4" t="n"/>
-      <c r="D81" s="4" t="n"/>
-      <c r="E81" s="4" t="n"/>
-      <c r="F81" s="4" t="n"/>
-      <c r="G81" s="4" t="n"/>
-      <c r="H81" s="4" t="n"/>
-      <c r="I81" s="4" t="n"/>
-      <c r="J81" s="4" t="n"/>
-      <c r="K81" s="4" t="n"/>
-      <c r="L81" s="4" t="n"/>
+      <c r="B81" s="27" t="n"/>
+      <c r="C81" s="27" t="n"/>
+      <c r="D81" s="27" t="n"/>
+      <c r="E81" s="27" t="n"/>
+      <c r="F81" s="27" t="n"/>
+      <c r="G81" s="27" t="n"/>
+      <c r="H81" s="27" t="n"/>
+      <c r="I81" s="27" t="n"/>
+      <c r="J81" s="27" t="n"/>
+      <c r="K81" s="27" t="n"/>
+      <c r="L81" s="28" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -2937,17 +2983,17 @@
           <t>8. TABLA DE AMORTIZACIÓN DEL PRÉSTAMO  (cuota anual fija)</t>
         </is>
       </c>
-      <c r="B88" s="4" t="n"/>
-      <c r="C88" s="4" t="n"/>
-      <c r="D88" s="4" t="n"/>
-      <c r="E88" s="4" t="n"/>
-      <c r="F88" s="4" t="n"/>
-      <c r="G88" s="4" t="n"/>
-      <c r="H88" s="4" t="n"/>
-      <c r="I88" s="4" t="n"/>
-      <c r="J88" s="4" t="n"/>
-      <c r="K88" s="4" t="n"/>
-      <c r="L88" s="4" t="n"/>
+      <c r="B88" s="27" t="n"/>
+      <c r="C88" s="27" t="n"/>
+      <c r="D88" s="27" t="n"/>
+      <c r="E88" s="27" t="n"/>
+      <c r="F88" s="27" t="n"/>
+      <c r="G88" s="27" t="n"/>
+      <c r="H88" s="27" t="n"/>
+      <c r="I88" s="27" t="n"/>
+      <c r="J88" s="27" t="n"/>
+      <c r="K88" s="27" t="n"/>
+      <c r="L88" s="28" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -3267,17 +3313,17 @@
           <t>9. FLUJO DE CAJA DEL PROYECTO (SIN FINANCIAMIENTO)</t>
         </is>
       </c>
-      <c r="B96" s="4" t="n"/>
-      <c r="C96" s="4" t="n"/>
-      <c r="D96" s="4" t="n"/>
-      <c r="E96" s="4" t="n"/>
-      <c r="F96" s="4" t="n"/>
-      <c r="G96" s="4" t="n"/>
-      <c r="H96" s="4" t="n"/>
-      <c r="I96" s="4" t="n"/>
-      <c r="J96" s="4" t="n"/>
-      <c r="K96" s="4" t="n"/>
-      <c r="L96" s="4" t="n"/>
+      <c r="B96" s="27" t="n"/>
+      <c r="C96" s="27" t="n"/>
+      <c r="D96" s="27" t="n"/>
+      <c r="E96" s="27" t="n"/>
+      <c r="F96" s="27" t="n"/>
+      <c r="G96" s="27" t="n"/>
+      <c r="H96" s="27" t="n"/>
+      <c r="I96" s="27" t="n"/>
+      <c r="J96" s="27" t="n"/>
+      <c r="K96" s="27" t="n"/>
+      <c r="L96" s="28" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -4088,17 +4134,17 @@
           <t>10. FLUJO DE CAJA DEL PROYECTO (CON FINANCIAMIENTO)</t>
         </is>
       </c>
-      <c r="B114" s="4" t="n"/>
-      <c r="C114" s="4" t="n"/>
-      <c r="D114" s="4" t="n"/>
-      <c r="E114" s="4" t="n"/>
-      <c r="F114" s="4" t="n"/>
-      <c r="G114" s="4" t="n"/>
-      <c r="H114" s="4" t="n"/>
-      <c r="I114" s="4" t="n"/>
-      <c r="J114" s="4" t="n"/>
-      <c r="K114" s="4" t="n"/>
-      <c r="L114" s="4" t="n"/>
+      <c r="B114" s="27" t="n"/>
+      <c r="C114" s="27" t="n"/>
+      <c r="D114" s="27" t="n"/>
+      <c r="E114" s="27" t="n"/>
+      <c r="F114" s="27" t="n"/>
+      <c r="G114" s="27" t="n"/>
+      <c r="H114" s="27" t="n"/>
+      <c r="I114" s="27" t="n"/>
+      <c r="J114" s="27" t="n"/>
+      <c r="K114" s="27" t="n"/>
+      <c r="L114" s="28" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -5050,17 +5096,17 @@
           <t>11. COSTO DE CAPITAL — PROYECTO PURO (sin financiamiento)</t>
         </is>
       </c>
-      <c r="B135" s="4" t="n"/>
-      <c r="C135" s="4" t="n"/>
-      <c r="D135" s="4" t="n"/>
-      <c r="E135" s="4" t="n"/>
-      <c r="F135" s="4" t="n"/>
-      <c r="G135" s="4" t="n"/>
-      <c r="H135" s="4" t="n"/>
-      <c r="I135" s="4" t="n"/>
-      <c r="J135" s="4" t="n"/>
-      <c r="K135" s="4" t="n"/>
-      <c r="L135" s="4" t="n"/>
+      <c r="B135" s="27" t="n"/>
+      <c r="C135" s="27" t="n"/>
+      <c r="D135" s="27" t="n"/>
+      <c r="E135" s="27" t="n"/>
+      <c r="F135" s="27" t="n"/>
+      <c r="G135" s="27" t="n"/>
+      <c r="H135" s="27" t="n"/>
+      <c r="I135" s="27" t="n"/>
+      <c r="J135" s="27" t="n"/>
+      <c r="K135" s="27" t="n"/>
+      <c r="L135" s="28" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
@@ -5148,17 +5194,17 @@
           <t>12. INDICADORES FINANCIEROS — PROYECTO PURO</t>
         </is>
       </c>
-      <c r="B140" s="4" t="n"/>
-      <c r="C140" s="4" t="n"/>
-      <c r="D140" s="4" t="n"/>
-      <c r="E140" s="4" t="n"/>
-      <c r="F140" s="4" t="n"/>
-      <c r="G140" s="4" t="n"/>
-      <c r="H140" s="4" t="n"/>
-      <c r="I140" s="4" t="n"/>
-      <c r="J140" s="4" t="n"/>
-      <c r="K140" s="4" t="n"/>
-      <c r="L140" s="4" t="n"/>
+      <c r="B140" s="27" t="n"/>
+      <c r="C140" s="27" t="n"/>
+      <c r="D140" s="27" t="n"/>
+      <c r="E140" s="27" t="n"/>
+      <c r="F140" s="27" t="n"/>
+      <c r="G140" s="27" t="n"/>
+      <c r="H140" s="27" t="n"/>
+      <c r="I140" s="27" t="n"/>
+      <c r="J140" s="27" t="n"/>
+      <c r="K140" s="27" t="n"/>
+      <c r="L140" s="28" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="21" t="inlineStr">
@@ -5174,11 +5220,11 @@
     <row r="142">
       <c r="A142" s="21" t="inlineStr">
         <is>
-          <t>TIR (Tasa Interna de Retorno)</t>
+          <t>TIRM (Tasa Interna de Retorno Modificada)</t>
         </is>
       </c>
       <c r="B142" s="7">
-        <f>IRR(B111:L111)</f>
+        <f>MIRR(B111:L111,E138,E138)</f>
         <v/>
       </c>
     </row>
@@ -5210,17 +5256,17 @@
           <t>13. COSTO DE CAPITAL — CON FINANCIAMIENTO (WACC)</t>
         </is>
       </c>
-      <c r="B146" s="4" t="n"/>
-      <c r="C146" s="4" t="n"/>
-      <c r="D146" s="4" t="n"/>
-      <c r="E146" s="4" t="n"/>
-      <c r="F146" s="4" t="n"/>
-      <c r="G146" s="4" t="n"/>
-      <c r="H146" s="4" t="n"/>
-      <c r="I146" s="4" t="n"/>
-      <c r="J146" s="4" t="n"/>
-      <c r="K146" s="4" t="n"/>
-      <c r="L146" s="4" t="n"/>
+      <c r="B146" s="27" t="n"/>
+      <c r="C146" s="27" t="n"/>
+      <c r="D146" s="27" t="n"/>
+      <c r="E146" s="27" t="n"/>
+      <c r="F146" s="27" t="n"/>
+      <c r="G146" s="27" t="n"/>
+      <c r="H146" s="27" t="n"/>
+      <c r="I146" s="27" t="n"/>
+      <c r="J146" s="27" t="n"/>
+      <c r="K146" s="27" t="n"/>
+      <c r="L146" s="28" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -5331,17 +5377,17 @@
           <t>14. INDICADORES FINANCIEROS — CON FINANCIAMIENTO</t>
         </is>
       </c>
-      <c r="B152" s="4" t="n"/>
-      <c r="C152" s="4" t="n"/>
-      <c r="D152" s="4" t="n"/>
-      <c r="E152" s="4" t="n"/>
-      <c r="F152" s="4" t="n"/>
-      <c r="G152" s="4" t="n"/>
-      <c r="H152" s="4" t="n"/>
-      <c r="I152" s="4" t="n"/>
-      <c r="J152" s="4" t="n"/>
-      <c r="K152" s="4" t="n"/>
-      <c r="L152" s="4" t="n"/>
+      <c r="B152" s="27" t="n"/>
+      <c r="C152" s="27" t="n"/>
+      <c r="D152" s="27" t="n"/>
+      <c r="E152" s="27" t="n"/>
+      <c r="F152" s="27" t="n"/>
+      <c r="G152" s="27" t="n"/>
+      <c r="H152" s="27" t="n"/>
+      <c r="I152" s="27" t="n"/>
+      <c r="J152" s="27" t="n"/>
+      <c r="K152" s="27" t="n"/>
+      <c r="L152" s="28" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="21" t="inlineStr">
@@ -5357,11 +5403,11 @@
     <row r="154">
       <c r="A154" s="21" t="inlineStr">
         <is>
-          <t>TIR (Tasa Interna de Retorno)</t>
+          <t>TIRM (Tasa Interna de Retorno Modificada)</t>
         </is>
       </c>
       <c r="B154" s="7">
-        <f>IRR(B132:L132)</f>
+        <f>MIRR(B132:L132,E150,E150)</f>
         <v/>
       </c>
     </row>
@@ -5393,17 +5439,17 @@
           <t>15. NOTAS LEGALES (cumplimiento normativo Honduras)</t>
         </is>
       </c>
-      <c r="B158" s="4" t="n"/>
-      <c r="C158" s="4" t="n"/>
-      <c r="D158" s="4" t="n"/>
-      <c r="E158" s="4" t="n"/>
-      <c r="F158" s="4" t="n"/>
-      <c r="G158" s="4" t="n"/>
-      <c r="H158" s="4" t="n"/>
-      <c r="I158" s="4" t="n"/>
-      <c r="J158" s="4" t="n"/>
-      <c r="K158" s="4" t="n"/>
-      <c r="L158" s="4" t="n"/>
+      <c r="B158" s="27" t="n"/>
+      <c r="C158" s="27" t="n"/>
+      <c r="D158" s="27" t="n"/>
+      <c r="E158" s="27" t="n"/>
+      <c r="F158" s="27" t="n"/>
+      <c r="G158" s="27" t="n"/>
+      <c r="H158" s="27" t="n"/>
+      <c r="I158" s="27" t="n"/>
+      <c r="J158" s="27" t="n"/>
+      <c r="K158" s="27" t="n"/>
+      <c r="L158" s="28" t="n"/>
     </row>
     <row r="159" ht="30" customHeight="1">
       <c r="A159" s="26" t="inlineStr">
@@ -5411,17 +5457,17 @@
           <t>• ISR: 25% + aportación solidaria 5% sobre el excedente de L 1,000,000 (Ley del ISR).</t>
         </is>
       </c>
-      <c r="B159" s="14" t="n"/>
-      <c r="C159" s="14" t="n"/>
-      <c r="D159" s="14" t="n"/>
-      <c r="E159" s="14" t="n"/>
-      <c r="F159" s="14" t="n"/>
-      <c r="G159" s="14" t="n"/>
-      <c r="H159" s="14" t="n"/>
-      <c r="I159" s="14" t="n"/>
-      <c r="J159" s="14" t="n"/>
-      <c r="K159" s="14" t="n"/>
-      <c r="L159" s="14" t="n"/>
+      <c r="B159" s="27" t="n"/>
+      <c r="C159" s="27" t="n"/>
+      <c r="D159" s="27" t="n"/>
+      <c r="E159" s="27" t="n"/>
+      <c r="F159" s="27" t="n"/>
+      <c r="G159" s="27" t="n"/>
+      <c r="H159" s="27" t="n"/>
+      <c r="I159" s="27" t="n"/>
+      <c r="J159" s="27" t="n"/>
+      <c r="K159" s="27" t="n"/>
+      <c r="L159" s="28" t="n"/>
     </row>
     <row r="160" ht="30" customHeight="1">
       <c r="A160" s="26" t="inlineStr">
@@ -5429,17 +5475,17 @@
           <t>• Depreciación línea recta: maquinaria 10%; vehículos 10%-33% (aquí 20% = 5 años); diferidos 5 años.</t>
         </is>
       </c>
-      <c r="B160" s="14" t="n"/>
-      <c r="C160" s="14" t="n"/>
-      <c r="D160" s="14" t="n"/>
-      <c r="E160" s="14" t="n"/>
-      <c r="F160" s="14" t="n"/>
-      <c r="G160" s="14" t="n"/>
-      <c r="H160" s="14" t="n"/>
-      <c r="I160" s="14" t="n"/>
-      <c r="J160" s="14" t="n"/>
-      <c r="K160" s="14" t="n"/>
-      <c r="L160" s="14" t="n"/>
+      <c r="B160" s="27" t="n"/>
+      <c r="C160" s="27" t="n"/>
+      <c r="D160" s="27" t="n"/>
+      <c r="E160" s="27" t="n"/>
+      <c r="F160" s="27" t="n"/>
+      <c r="G160" s="27" t="n"/>
+      <c r="H160" s="27" t="n"/>
+      <c r="I160" s="27" t="n"/>
+      <c r="J160" s="27" t="n"/>
+      <c r="K160" s="27" t="n"/>
+      <c r="L160" s="28" t="n"/>
     </row>
     <row r="161" ht="30" customHeight="1">
       <c r="A161" s="26" t="inlineStr">
@@ -5447,17 +5493,17 @@
           <t>• Seguridad social patronal (techo L 11,903.13): IHSS EM 2.5% + IVM 1% + RP 0.2% + RAP 1.5%; INFOP 1% sobre planilla (sin techo).</t>
         </is>
       </c>
-      <c r="B161" s="14" t="n"/>
-      <c r="C161" s="14" t="n"/>
-      <c r="D161" s="14" t="n"/>
-      <c r="E161" s="14" t="n"/>
-      <c r="F161" s="14" t="n"/>
-      <c r="G161" s="14" t="n"/>
-      <c r="H161" s="14" t="n"/>
-      <c r="I161" s="14" t="n"/>
-      <c r="J161" s="14" t="n"/>
-      <c r="K161" s="14" t="n"/>
-      <c r="L161" s="14" t="n"/>
+      <c r="B161" s="27" t="n"/>
+      <c r="C161" s="27" t="n"/>
+      <c r="D161" s="27" t="n"/>
+      <c r="E161" s="27" t="n"/>
+      <c r="F161" s="27" t="n"/>
+      <c r="G161" s="27" t="n"/>
+      <c r="H161" s="27" t="n"/>
+      <c r="I161" s="27" t="n"/>
+      <c r="J161" s="27" t="n"/>
+      <c r="K161" s="27" t="n"/>
+      <c r="L161" s="28" t="n"/>
     </row>
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="26" t="inlineStr">
@@ -5465,17 +5511,17 @@
           <t>• Prestaciones: aguinaldo (13.º mes) y catorceavo (14.º mes) — Código del Trabajo.</t>
         </is>
       </c>
-      <c r="B162" s="14" t="n"/>
-      <c r="C162" s="14" t="n"/>
-      <c r="D162" s="14" t="n"/>
-      <c r="E162" s="14" t="n"/>
-      <c r="F162" s="14" t="n"/>
-      <c r="G162" s="14" t="n"/>
-      <c r="H162" s="14" t="n"/>
-      <c r="I162" s="14" t="n"/>
-      <c r="J162" s="14" t="n"/>
-      <c r="K162" s="14" t="n"/>
-      <c r="L162" s="14" t="n"/>
+      <c r="B162" s="27" t="n"/>
+      <c r="C162" s="27" t="n"/>
+      <c r="D162" s="27" t="n"/>
+      <c r="E162" s="27" t="n"/>
+      <c r="F162" s="27" t="n"/>
+      <c r="G162" s="27" t="n"/>
+      <c r="H162" s="27" t="n"/>
+      <c r="I162" s="27" t="n"/>
+      <c r="J162" s="27" t="n"/>
+      <c r="K162" s="27" t="n"/>
+      <c r="L162" s="28" t="n"/>
     </row>
     <row r="163" ht="30" customHeight="1">
       <c r="A163" s="26" t="inlineStr">
@@ -5483,17 +5529,17 @@
           <t>• ISV: la leche fluida/pasteurizada está exenta; no se cobra ISV en ventas.</t>
         </is>
       </c>
-      <c r="B163" s="14" t="n"/>
-      <c r="C163" s="14" t="n"/>
-      <c r="D163" s="14" t="n"/>
-      <c r="E163" s="14" t="n"/>
-      <c r="F163" s="14" t="n"/>
-      <c r="G163" s="14" t="n"/>
-      <c r="H163" s="14" t="n"/>
-      <c r="I163" s="14" t="n"/>
-      <c r="J163" s="14" t="n"/>
-      <c r="K163" s="14" t="n"/>
-      <c r="L163" s="14" t="n"/>
+      <c r="B163" s="27" t="n"/>
+      <c r="C163" s="27" t="n"/>
+      <c r="D163" s="27" t="n"/>
+      <c r="E163" s="27" t="n"/>
+      <c r="F163" s="27" t="n"/>
+      <c r="G163" s="27" t="n"/>
+      <c r="H163" s="27" t="n"/>
+      <c r="I163" s="27" t="n"/>
+      <c r="J163" s="27" t="n"/>
+      <c r="K163" s="27" t="n"/>
+      <c r="L163" s="28" t="n"/>
     </row>
     <row r="164" ht="30" customHeight="1">
       <c r="A164" s="26" t="inlineStr">
@@ -5501,17 +5547,17 @@
           <t>• Arrastre de pérdidas fiscales: la manufactura puede compensarlas hasta 3 años (aplicado en el flujo, línea de pérdidas acumuladas).</t>
         </is>
       </c>
-      <c r="B164" s="14" t="n"/>
-      <c r="C164" s="14" t="n"/>
-      <c r="D164" s="14" t="n"/>
-      <c r="E164" s="14" t="n"/>
-      <c r="F164" s="14" t="n"/>
-      <c r="G164" s="14" t="n"/>
-      <c r="H164" s="14" t="n"/>
-      <c r="I164" s="14" t="n"/>
-      <c r="J164" s="14" t="n"/>
-      <c r="K164" s="14" t="n"/>
-      <c r="L164" s="14" t="n"/>
+      <c r="B164" s="27" t="n"/>
+      <c r="C164" s="27" t="n"/>
+      <c r="D164" s="27" t="n"/>
+      <c r="E164" s="27" t="n"/>
+      <c r="F164" s="27" t="n"/>
+      <c r="G164" s="27" t="n"/>
+      <c r="H164" s="27" t="n"/>
+      <c r="I164" s="27" t="n"/>
+      <c r="J164" s="27" t="n"/>
+      <c r="K164" s="27" t="n"/>
+      <c r="L164" s="28" t="n"/>
     </row>
     <row r="165" ht="30" customHeight="1">
       <c r="A165" s="26" t="inlineStr">
@@ -5519,17 +5565,17 @@
           <t>• Impuesto al Activo Neto 1% (deducción L3M; exento en preoperación; se paga solo si supera al ISR).</t>
         </is>
       </c>
-      <c r="B165" s="14" t="n"/>
-      <c r="C165" s="14" t="n"/>
-      <c r="D165" s="14" t="n"/>
-      <c r="E165" s="14" t="n"/>
-      <c r="F165" s="14" t="n"/>
-      <c r="G165" s="14" t="n"/>
-      <c r="H165" s="14" t="n"/>
-      <c r="I165" s="14" t="n"/>
-      <c r="J165" s="14" t="n"/>
-      <c r="K165" s="14" t="n"/>
-      <c r="L165" s="14" t="n"/>
+      <c r="B165" s="27" t="n"/>
+      <c r="C165" s="27" t="n"/>
+      <c r="D165" s="27" t="n"/>
+      <c r="E165" s="27" t="n"/>
+      <c r="F165" s="27" t="n"/>
+      <c r="G165" s="27" t="n"/>
+      <c r="H165" s="27" t="n"/>
+      <c r="I165" s="27" t="n"/>
+      <c r="J165" s="27" t="n"/>
+      <c r="K165" s="27" t="n"/>
+      <c r="L165" s="28" t="n"/>
     </row>
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="26" t="inlineStr">
@@ -5537,17 +5583,17 @@
           <t>• Capital de trabajo: 1 mes de costos operativos, financiado con crédito de proveedores (CREL/ganaderos).</t>
         </is>
       </c>
-      <c r="B166" s="14" t="n"/>
-      <c r="C166" s="14" t="n"/>
-      <c r="D166" s="14" t="n"/>
-      <c r="E166" s="14" t="n"/>
-      <c r="F166" s="14" t="n"/>
-      <c r="G166" s="14" t="n"/>
-      <c r="H166" s="14" t="n"/>
-      <c r="I166" s="14" t="n"/>
-      <c r="J166" s="14" t="n"/>
-      <c r="K166" s="14" t="n"/>
-      <c r="L166" s="14" t="n"/>
+      <c r="B166" s="27" t="n"/>
+      <c r="C166" s="27" t="n"/>
+      <c r="D166" s="27" t="n"/>
+      <c r="E166" s="27" t="n"/>
+      <c r="F166" s="27" t="n"/>
+      <c r="G166" s="27" t="n"/>
+      <c r="H166" s="27" t="n"/>
+      <c r="I166" s="27" t="n"/>
+      <c r="J166" s="27" t="n"/>
+      <c r="K166" s="27" t="n"/>
+      <c r="L166" s="28" t="n"/>
     </row>
     <row r="167" ht="30" customHeight="1">
       <c r="A167" s="26" t="inlineStr">
@@ -5555,17 +5601,17 @@
           <t>• Impuestos municipales de Comayagua (industria, comercio y servicios; bienes inmuebles).</t>
         </is>
       </c>
-      <c r="B167" s="14" t="n"/>
-      <c r="C167" s="14" t="n"/>
-      <c r="D167" s="14" t="n"/>
-      <c r="E167" s="14" t="n"/>
-      <c r="F167" s="14" t="n"/>
-      <c r="G167" s="14" t="n"/>
-      <c r="H167" s="14" t="n"/>
-      <c r="I167" s="14" t="n"/>
-      <c r="J167" s="14" t="n"/>
-      <c r="K167" s="14" t="n"/>
-      <c r="L167" s="14" t="n"/>
+      <c r="B167" s="27" t="n"/>
+      <c r="C167" s="27" t="n"/>
+      <c r="D167" s="27" t="n"/>
+      <c r="E167" s="27" t="n"/>
+      <c r="F167" s="27" t="n"/>
+      <c r="G167" s="27" t="n"/>
+      <c r="H167" s="27" t="n"/>
+      <c r="I167" s="27" t="n"/>
+      <c r="J167" s="27" t="n"/>
+      <c r="K167" s="27" t="n"/>
+      <c r="L167" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="34">

</xml_diff>

<commit_message>
Precio de venta indexado a inflacion 4.5% (igual que costos) para consistencia de margen real; Excel y tesis actualizados (VAN/TIRM/PRI/Cuadro 1)
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -1297,7 +1297,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Precio de venta (Lps/litro)</t>
+          <t>Precio de venta (Lps/litro) — base 28 indexado a inflación 4.5%</t>
         </is>
       </c>
       <c r="B41" s="12" t="n">
@@ -1306,32 +1306,41 @@
       <c r="C41" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="D41" s="12" t="n">
-        <v>29</v>
-      </c>
-      <c r="E41" s="12" t="n">
-        <v>30</v>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>31</v>
-      </c>
-      <c r="G41" s="12" t="n">
-        <v>32</v>
-      </c>
-      <c r="H41" s="12" t="n">
-        <v>33</v>
-      </c>
-      <c r="I41" s="12" t="n">
-        <v>34</v>
-      </c>
-      <c r="J41" s="12" t="n">
-        <v>35</v>
-      </c>
-      <c r="K41" s="12" t="n">
-        <v>36</v>
-      </c>
-      <c r="L41" s="12" t="n">
-        <v>37</v>
+      <c r="D41" s="12">
+        <f>C41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="E41" s="12">
+        <f>D41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="F41" s="12">
+        <f>E41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="G41" s="12">
+        <f>F41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="H41" s="12">
+        <f>G41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="I41" s="12">
+        <f>H41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="J41" s="12">
+        <f>I41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="K41" s="12">
+        <f>J41*(1+$B$11)</f>
+        <v/>
+      </c>
+      <c r="L41" s="12">
+        <f>K41*(1+$B$11)</f>
+        <v/>
       </c>
     </row>
     <row r="42">

</xml_diff>

<commit_message>
Excel: titulo limpio (Estudio Financiero del Proyecto + nombre del proyecto) y elimina hoja de Correcciones ya aplicadas en ambos documentos
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estudio Financiero" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correcciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -581,14 +580,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PRODUCTORA DE LECHE PASTEURIZADA «PURA» — Flujo de Caja del Proyecto</t>
+          <t>Estudio Financiero del Proyecto</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Estudio financiero conforme a la normativa de Honduras · cifras en Lempiras · toda celda de resultado es fórmula</t>
+          <t>Productora de Leche Pasteurizada «Pura»</t>
         </is>
       </c>
     </row>
@@ -5661,293 +5660,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>Correcciones a realizar en el documento de tesis</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Dónde en la tesis</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Qué está mal</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Corrección</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="26" t="inlineStr">
-        <is>
-          <t>Cuadro 6 / Costo de personal</t>
-        </is>
-      </c>
-      <c r="C3" s="26" t="inlineStr">
-        <is>
-          <t>Planilla mensual (L92,600) usada como costo anual</t>
-        </is>
-      </c>
-      <c r="D3" s="26" t="inlineStr">
-        <is>
-          <t>Anualizar ×12 + aguinaldo + catorceavo + cargas patronales con techo</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="42" customHeight="1">
-      <c r="A4" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="26" t="inlineStr">
-        <is>
-          <t>Cuadros 5 y 6</t>
-        </is>
-      </c>
-      <c r="C4" s="26" t="inlineStr">
-        <is>
-          <t>Personal contado dos veces</t>
-        </is>
-      </c>
-      <c r="D4" s="26" t="inlineStr">
-        <is>
-          <t>Dejarlo en una sola línea</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="26" t="inlineStr">
-        <is>
-          <t>Cuadros 5 y 6</t>
-        </is>
-      </c>
-      <c r="C5" s="26" t="inlineStr">
-        <is>
-          <t>Costos mensuales usados como anuales</t>
-        </is>
-      </c>
-      <c r="D5" s="26" t="inlineStr">
-        <is>
-          <t>Multiplicar por 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>Costos fijos (leche L390,000)</t>
-        </is>
-      </c>
-      <c r="C6" s="26" t="inlineStr">
-        <is>
-          <t>Leche, empaque y combustible como fijos</t>
-        </is>
-      </c>
-      <c r="D6" s="26" t="inlineStr">
-        <is>
-          <t>Volverlos variables (por litro vendido)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="26" t="inlineStr">
-        <is>
-          <t>Gastos administrativos</t>
-        </is>
-      </c>
-      <c r="C7" s="26" t="inlineStr">
-        <is>
-          <t>Suman L21,600 pero dice L22,600</t>
-        </is>
-      </c>
-      <c r="D7" s="26" t="inlineStr">
-        <is>
-          <t>Corregir la suma</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" s="26" t="inlineStr">
-        <is>
-          <t>Cuadro 3 (depreciación)</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>Camión con vida de 3 años</t>
-        </is>
-      </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>Vida útil 5 años (rango legal 10-33%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="26" t="inlineStr">
-        <is>
-          <t>Estudio financiero</t>
-        </is>
-      </c>
-      <c r="C9" s="26" t="inlineStr">
-        <is>
-          <t>No aplica ISR</t>
-        </is>
-      </c>
-      <c r="D9" s="26" t="inlineStr">
-        <is>
-          <t>ISR 25% + 5% solidaria (renta &gt; L1M)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="26" t="inlineStr">
-        <is>
-          <t>Estudio financiero</t>
-        </is>
-      </c>
-      <c r="C10" s="26" t="inlineStr">
-        <is>
-          <t>No define tasa de descuento ni WACC</t>
-        </is>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
-        <is>
-          <t>Tasa de descuento 15% y WACC calculado</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="26" t="inlineStr">
-        <is>
-          <t>Estudio financiero</t>
-        </is>
-      </c>
-      <c r="C11" s="26" t="inlineStr">
-        <is>
-          <t>No incluye capital de trabajo</t>
-        </is>
-      </c>
-      <c r="D11" s="26" t="inlineStr">
-        <is>
-          <t>1 mes de costos (crédito proveedores), recuperado Año 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>Estudio financiero</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>No aprovecha arrastre de pérdidas</t>
-        </is>
-      </c>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>Compensar pérdidas de años iniciales (ley, 3 años)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>Estudio de personal</t>
-        </is>
-      </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>Faltan cargas sociales de ley</t>
-        </is>
-      </c>
-      <c r="D13" s="26" t="inlineStr">
-        <is>
-          <t>IHSS+RAP (con techo)+INFOP+aguinaldo+catorceavo</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="26" t="inlineStr">
-        <is>
-          <t>Cuadro 1 / ventas</t>
-        </is>
-      </c>
-      <c r="C14" s="26" t="inlineStr">
-        <is>
-          <t>Captación lenta (15 clientes)</t>
-        </is>
-      </c>
-      <c r="D14" s="26" t="inlineStr">
-        <is>
-          <t>Captación agresiva (60→690 clientes), consumo 150 L/mes</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: elimina guiones largos y textos redundantes (spell-outs de VAN/TIRM/PRI, descripciones de formula), y agrega hoja 'Explicacion del estudio'
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estudio Financiero" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación del estudio" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +35,23 @@
     <font>
       <name val="Calibri"/>
       <color rgb="FF000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -125,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -195,6 +213,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1032,7 +1059,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Gastos diferidos (preoperativos + legales)</t>
+          <t>Gastos diferidos preoperativos y legales</t>
         </is>
       </c>
       <c r="B33" s="12" t="n">
@@ -1126,7 +1153,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>2. PRODUCCIÓN Y VENTAS  (volumen = clientes × consumo mensual × 12)</t>
+          <t>2. PRODUCCIÓN Y VENTAS</t>
         </is>
       </c>
       <c r="B37" s="27" t="n"/>
@@ -1296,7 +1323,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>Precio de venta (Lps/litro) — base 28 indexado a inflación 4.5%</t>
+          <t>Precio de venta (Lps/litro)</t>
         </is>
       </c>
       <c r="B41" s="12" t="n">
@@ -1345,7 +1372,7 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>INGRESOS POR VENTAS  (= volumen × precio; leche exenta de ISV)</t>
+          <t>INGRESOS POR VENTAS</t>
         </is>
       </c>
       <c r="B42" s="16">
@@ -1396,7 +1423,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>3. COSTOS VARIABLES  (= litros × costo unitario × inflación)</t>
+          <t>3. COSTOS VARIABLES</t>
         </is>
       </c>
       <c r="B44" s="27" t="n"/>
@@ -1677,7 +1704,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>4. COSTO DE PERSONAL  (con prestaciones y seguridad social de ley)</t>
+          <t>4. COSTO DE PERSONAL</t>
         </is>
       </c>
       <c r="B51" s="27" t="n"/>
@@ -1859,7 +1886,7 @@
     <row r="59">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>Planilla mensual total  /  base cotizable total</t>
+          <t>Planilla mensual y base cotizable</t>
         </is>
       </c>
       <c r="B59" s="16">
@@ -1883,7 +1910,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Cargas patronales mensuales  (base cotizable × 5.2% + planilla × 1% INFOP)</t>
+          <t>Cargas patronales mensuales</t>
         </is>
       </c>
       <c r="B60" s="12">
@@ -1966,7 +1993,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>Costo anual de personal  (planilla × 14 meses + cargas patronales × 12)</t>
+          <t>Costo anual de personal</t>
         </is>
       </c>
       <c r="B62" s="12" t="n">
@@ -2096,7 +2123,7 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>Costos fijos operativos (mensual × 12 × inflación)</t>
+          <t>Costos fijos operativos</t>
         </is>
       </c>
       <c r="B66" s="12" t="n">
@@ -2146,7 +2173,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>Gastos administrativos (mensual × 12 × inflación)</t>
+          <t>Gastos administrativos</t>
         </is>
       </c>
       <c r="B67" s="12" t="n">
@@ -2196,7 +2223,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>Personal (de la sección 4)</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B68" s="12">
@@ -2298,7 +2325,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>6. DEPRECIACIONES Y AMORTIZACIONES  (línea recta = Valor ÷ Vida)</t>
+          <t>6. DEPRECIACIONES Y AMORTIZACIONES</t>
         </is>
       </c>
       <c r="B71" s="27" t="n"/>
@@ -2845,7 +2872,7 @@
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>Capital de trabajo requerido (= (variables+fijos) × meses ÷ 12)</t>
+          <t>Capital de trabajo requerido</t>
         </is>
       </c>
       <c r="B84" s="12">
@@ -2988,7 +3015,7 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>8. TABLA DE AMORTIZACIÓN DEL PRÉSTAMO  (cuota anual fija)</t>
+          <t>8. TABLA DE AMORTIZACIÓN DEL PRÉSTAMO</t>
         </is>
       </c>
       <c r="B88" s="27" t="n"/>
@@ -3168,7 +3195,7 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>Intereses (= saldo × tasa)</t>
+          <t>Intereses</t>
         </is>
       </c>
       <c r="B92" s="12" t="n">
@@ -3218,7 +3245,7 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>Cuota total (= abono + intereses)</t>
+          <t>Cuota total</t>
         </is>
       </c>
       <c r="B93" s="12" t="n">
@@ -3652,7 +3679,7 @@
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>Pérdidas fiscales acumuladas (arrastre 3 años, manufactura)</t>
+          <t>Pérdidas fiscales acumuladas</t>
         </is>
       </c>
       <c r="B103" s="12" t="n">
@@ -3702,7 +3729,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>(−) Impuesto sobre la renta (25% + 5% solidaria, neto de pérdidas)</t>
+          <t>(−) Impuesto sobre la renta</t>
         </is>
       </c>
       <c r="B104" s="12" t="n">
@@ -4372,7 +4399,7 @@
     <row r="119">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>(−) Gastos financieros (intereses)</t>
+          <t>(−) Gastos financieros</t>
         </is>
       </c>
       <c r="B119" s="12" t="n">
@@ -4523,7 +4550,7 @@
     <row r="122">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>Pérdidas fiscales acumuladas (arrastre 3 años, manufactura)</t>
+          <t>Pérdidas fiscales acumuladas</t>
         </is>
       </c>
       <c r="B122" s="12" t="n">
@@ -4573,7 +4600,7 @@
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>(−) Impuesto sobre la renta (25% + 5% solidaria, neto de pérdidas)</t>
+          <t>(−) Impuesto sobre la renta</t>
         </is>
       </c>
       <c r="B123" s="12" t="n">
@@ -5101,7 +5128,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>11. COSTO DE CAPITAL — PROYECTO PURO (sin financiamiento)</t>
+          <t>11. COSTO DE CAPITAL DEL PROYECTO PURO</t>
         </is>
       </c>
       <c r="B135" s="27" t="n"/>
@@ -5153,7 +5180,7 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>Recursos propios (100%)</t>
+          <t>Recursos propios</t>
         </is>
       </c>
       <c r="B137" s="12">
@@ -5176,7 +5203,7 @@
     <row r="138">
       <c r="A138" s="15" t="inlineStr">
         <is>
-          <t>TOTAL / Tasa de descuento del proyecto</t>
+          <t>Tasa de descuento del proyecto</t>
         </is>
       </c>
       <c r="B138" s="16">
@@ -5199,7 +5226,7 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>12. INDICADORES FINANCIEROS — PROYECTO PURO</t>
+          <t>12. INDICADORES FINANCIEROS DEL PROYECTO PURO</t>
         </is>
       </c>
       <c r="B140" s="27" t="n"/>
@@ -5217,7 +5244,7 @@
     <row r="141">
       <c r="A141" s="21" t="inlineStr">
         <is>
-          <t>VAN (Valor Actual Neto)</t>
+          <t>VAN</t>
         </is>
       </c>
       <c r="B141" s="8">
@@ -5228,7 +5255,7 @@
     <row r="142">
       <c r="A142" s="21" t="inlineStr">
         <is>
-          <t>TIRM (Tasa Interna de Retorno Modificada)</t>
+          <t>TIRM</t>
         </is>
       </c>
       <c r="B142" s="7">
@@ -5239,7 +5266,7 @@
     <row r="143">
       <c r="A143" s="21" t="inlineStr">
         <is>
-          <t>PRI (años de recuperación)</t>
+          <t>PRI (años)</t>
         </is>
       </c>
       <c r="B143" s="9">
@@ -5261,7 +5288,7 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>13. COSTO DE CAPITAL — CON FINANCIAMIENTO (WACC)</t>
+          <t>13. COSTO DE CAPITAL CON FINANCIAMIENTO (WACC)</t>
         </is>
       </c>
       <c r="B146" s="27" t="n"/>
@@ -5313,7 +5340,7 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>Préstamo bancario (deuda, después de impuestos)</t>
+          <t>Préstamo bancario</t>
         </is>
       </c>
       <c r="B148" s="12">
@@ -5336,7 +5363,7 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>Recursos propios (patrimonio)</t>
+          <t>Recursos propios</t>
         </is>
       </c>
       <c r="B149" s="12">
@@ -5359,7 +5386,7 @@
     <row r="150">
       <c r="A150" s="15" t="inlineStr">
         <is>
-          <t>TOTAL / WACC</t>
+          <t>WACC</t>
         </is>
       </c>
       <c r="B150" s="16">
@@ -5382,7 +5409,7 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>14. INDICADORES FINANCIEROS — CON FINANCIAMIENTO</t>
+          <t>14. INDICADORES FINANCIEROS CON FINANCIAMIENTO</t>
         </is>
       </c>
       <c r="B152" s="27" t="n"/>
@@ -5400,7 +5427,7 @@
     <row r="153">
       <c r="A153" s="21" t="inlineStr">
         <is>
-          <t>VAN (Valor Actual Neto)</t>
+          <t>VAN</t>
         </is>
       </c>
       <c r="B153" s="8">
@@ -5411,7 +5438,7 @@
     <row r="154">
       <c r="A154" s="21" t="inlineStr">
         <is>
-          <t>TIRM (Tasa Interna de Retorno Modificada)</t>
+          <t>TIRM</t>
         </is>
       </c>
       <c r="B154" s="7">
@@ -5422,7 +5449,7 @@
     <row r="155">
       <c r="A155" s="21" t="inlineStr">
         <is>
-          <t>PRI (años de recuperación)</t>
+          <t>PRI (años)</t>
         </is>
       </c>
       <c r="B155" s="9">
@@ -5516,7 +5543,7 @@
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="26" t="inlineStr">
         <is>
-          <t>• Prestaciones: aguinaldo (13.º mes) y catorceavo (14.º mes) — Código del Trabajo.</t>
+          <t>• Prestaciones: aguinaldo (13.º mes) y catorceavo (14.º mes), Código del Trabajo.</t>
         </is>
       </c>
       <c r="B162" s="27" t="n"/>
@@ -5660,4 +5687,214 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="118" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Explicación del Estudio Financiero</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Productora de Leche Pasteurizada «Pura»</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="31" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>El estudio mide si conviene montar la planta de leche pasteurizada Pura. Proyecta los ingresos, los costos y el flujo de caja del proyecto durante diez años y calcula los indicadores de rentabilidad en dos escenarios: financiado con recursos propios y financiado con préstamo bancario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="31" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>Supuestos base</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Todas las cifras están en Lempiras. La inflación anual es de 4.5% y se aplica por igual a los precios de venta y a los costos, para que el margen del negocio no se distorsione. El impuesto sobre la renta es de 25%, más una aportación solidaria de 5% sobre la parte de la utilidad que supera un millón de Lempiras. El proyecto se financia mitad con préstamo bancario al 14% anual y mitad con recursos propios. La tasa de descuento del proyecto puro es de 15% y el costo promedio ponderado de capital del escenario con financiamiento es de 12.75%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="31" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Cómo se construye el estudio</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>1. Plan de inversiones. Reúne la maquinaria, el camión, los gastos diferidos y el capital de trabajo inicial. La inversión total es de 1,782,858 Lempiras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>2. Producción y ventas. El volumen se obtiene multiplicando los clientes por el consumo mensual de 150 litros y por 12 meses. El precio parte de 28 Lempiras por litro y sube cada año con la inflación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>3. Costos variables. Incluyen la leche cruda con merma, el empaque y el combustible de reparto. Crecen con el volumen y con la inflación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>4. Costo de personal. Seis puestos con salario, aguinaldo, catorceavo mes y las cargas de seguridad social calculadas sobre el techo de cotización de ley.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>5. Costos fijos. Reúnen los costos fijos operativos, los gastos administrativos y el personal, todos ajustados por inflación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>6. Depreciación y amortización. Se calcula por línea recta. La maquinaria se deprecia en diez años, el camión en cinco años y los gastos diferidos se amortizan en cinco años.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>7. Valor de desecho y capital de trabajo. El capital de trabajo equivale a un mes de costos operativos y se recupera en el último año.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>8. Amortización del préstamo. Muestra la cuota anual fija, los intereses y los abonos a capital del préstamo bancario a cinco años.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>9 y 10. Flujo de caja. Arma el flujo del proyecto sin financiamiento y con financiamiento. A la utilidad se le restan los impuestos, aprovechando el arrastre de pérdidas de los primeros años, y se le suman las partidas que no son salida de efectivo, como la depreciación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>11 a 14. Costo de capital e indicadores. Con la tasa de descuento y el WACC se calculan el VAN, la TIRM, el período de recuperación y la relación beneficio/costo en los dos escenarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>Qué significan los indicadores</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>El VAN es el valor de hoy de todo el efectivo que deja el proyecto después de cubrir la inversión; si es positivo, el proyecto crea valor. La TIRM es el rendimiento anual del proyecto suponiendo que las ganancias se reinvierten al costo de capital, por lo que resulta más realista que la TIR simple. El PRI es el tiempo, en años, que tarda en recuperarse la inversión. La relación beneficio/costo compara el valor presente de los ingresos con el de los egresos; si es mayor que uno, conviene invertir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Resultados</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>Proyecto puro: VAN de 15,452,178 Lempiras, TIRM de 40.52%, recuperación en 3.65 años y relación beneficio/costo de 1.23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Con financiamiento: VAN de 18,350,392 Lempiras, TIRM de 42.71%, recuperación en 3.63 años y relación beneficio/costo de 1.24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>En los dos escenarios el proyecto recupera la inversión antes de cuatro años y rinde por encima de la tasa exigida, por lo que es financieramente viable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Cumplimiento legal en Honduras</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>El estudio aplica el impuesto sobre la renta de 25% más 5% de aportación solidaria, la depreciación por línea recta permitida por el reglamento (vehículos entre 10% y 33%, aquí 20%), la seguridad social patronal con su techo de cotización, el aguinaldo y el catorceavo mes del Código del Trabajo, la exención del impuesto sobre ventas para la leche fluida, el arrastre de pérdidas de hasta tres años para la manufactura y los impuestos municipales de Comayagua.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Excel: reemplaza 'proyecto puro' por 'sin financiamiento' en encabezados y hoja de explicacion
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -5128,7 +5128,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>11. COSTO DE CAPITAL DEL PROYECTO PURO</t>
+          <t>11. COSTO DE CAPITAL SIN FINANCIAMIENTO</t>
         </is>
       </c>
       <c r="B135" s="27" t="n"/>
@@ -5226,7 +5226,7 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>12. INDICADORES FINANCIEROS DEL PROYECTO PURO</t>
+          <t>12. INDICADORES FINANCIEROS SIN FINANCIAMIENTO</t>
         </is>
       </c>
       <c r="B140" s="27" t="n"/>
@@ -5745,7 +5745,7 @@
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
         <is>
-          <t>Todas las cifras están en Lempiras. La inflación anual es de 4.5% y se aplica por igual a los precios de venta y a los costos, para que el margen del negocio no se distorsione. El impuesto sobre la renta es de 25%, más una aportación solidaria de 5% sobre la parte de la utilidad que supera un millón de Lempiras. El proyecto se financia mitad con préstamo bancario al 14% anual y mitad con recursos propios. La tasa de descuento del proyecto puro es de 15% y el costo promedio ponderado de capital del escenario con financiamiento es de 12.75%.</t>
+          <t>Todas las cifras están en Lempiras. La inflación anual es de 4.5% y se aplica por igual a los precios de venta y a los costos, para que el margen del negocio no se distorsione. El impuesto sobre la renta es de 25%, más una aportación solidaria de 5% sobre la parte de la utilidad que supera un millón de Lempiras. El proyecto se financia mitad con préstamo bancario al 14% anual y mitad con recursos propios. La tasa de descuento del escenario sin financiamiento es de 15% y el costo promedio ponderado de capital del escenario con financiamiento es de 12.75%.</t>
         </is>
       </c>
     </row>
@@ -5859,7 +5859,7 @@
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
         <is>
-          <t>Proyecto puro: VAN de 15,452,178 Lempiras, TIRM de 40.52%, recuperación en 3.65 años y relación beneficio/costo de 1.23.</t>
+          <t>Sin financiamiento: VAN de 15,452,178 Lempiras, TIRM de 40.52%, recuperación en 3.65 años y relación beneficio/costo de 1.23.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige seguridad social patronal a la ley HN: IHSS 7.2% (EM 5%+IVM 2%+RP 0.2%) sobre techo oficial L11,109.36, en vez del 5.2% erroneo; actualiza costos de personal, inversion y resultados en Excel y tesis (Cuadros 5 y 6)
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -773,11 +773,11 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Aporte patronal con techo (IHSS EM 2.5%+IVM 1%+RP 0.2%+RAP 1.5%)</t>
+          <t>Aporte patronal IHSS con techo (EM 5% + IVM 2% + RP 0.2%)</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>0.052</v>
+        <v>0.07199999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -793,11 +793,11 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Techo mensual de cotización IHSS/RAP (Lps)</t>
+          <t>Techo mensual de cotización IHSS (Lps)</t>
         </is>
       </c>
       <c r="B20" s="11" t="n">
-        <v>11903.13</v>
+        <v>11109.36</v>
       </c>
     </row>
     <row r="21">
@@ -5525,7 +5525,7 @@
     <row r="161" ht="30" customHeight="1">
       <c r="A161" s="26" t="inlineStr">
         <is>
-          <t>• Seguridad social patronal (techo L 11,903.13): IHSS EM 2.5% + IVM 1% + RP 0.2% + RAP 1.5%; INFOP 1% sobre planilla (sin techo).</t>
+          <t>• Seguridad social patronal (techo L 11,109.36): IHSS EM 5% + IVM 2% + RP 0.2% = 7.2%; INFOP 1% sobre planilla sin techo. El RAP (1.5%) es opcional desde el fallo de 2022.</t>
         </is>
       </c>
       <c r="B161" s="27" t="n"/>
@@ -5762,7 +5762,7 @@
     <row r="11">
       <c r="A11" s="31" t="inlineStr">
         <is>
-          <t>1. Plan de inversiones. Reúne la maquinaria, el camión, los gastos diferidos y el capital de trabajo inicial. La inversión total es de 1,782,858 Lempiras.</t>
+          <t>1. Plan de inversiones. Reúne la maquinaria, el camión, los gastos diferidos y el capital de trabajo inicial. La inversión total es de 1,784,058 Lempiras.</t>
         </is>
       </c>
     </row>
@@ -5859,14 +5859,14 @@
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
         <is>
-          <t>Sin financiamiento: VAN de 15,452,178 Lempiras, TIRM de 40.52%, recuperación en 3.65 años y relación beneficio/costo de 1.23.</t>
+          <t>Sin financiamiento: VAN de 15,389,173 Lempiras, TIRM de 40.40%, recuperación en 3.67 años y relación beneficio/costo de 1.23.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
         <is>
-          <t>Con financiamiento: VAN de 18,350,392 Lempiras, TIRM de 42.71%, recuperación en 3.63 años y relación beneficio/costo de 1.24.</t>
+          <t>Con financiamiento: VAN de 18,282,159 Lempiras, TIRM de 42.49%, recuperación en 3.66 años y relación beneficio/costo de 1.24.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: agrega impuesto municipal de Comayagua (ICS sobre ingresos, escala Art.78 Ley de Municipalidades) como linea deducible en el flujo; actualiza resultados en hoja de explicacion
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L167"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -3632,47 +3632,47 @@
         </is>
       </c>
       <c r="B102" s="16">
-        <f>B98-B99-B100-B101</f>
+        <f>B98-B99-B100-B101-B170</f>
         <v/>
       </c>
       <c r="C102" s="16">
-        <f>C98-C99-C100-C101</f>
+        <f>C98-C99-C100-C101-C170</f>
         <v/>
       </c>
       <c r="D102" s="16">
-        <f>D98-D99-D100-D101</f>
+        <f>D98-D99-D100-D101-D170</f>
         <v/>
       </c>
       <c r="E102" s="16">
-        <f>E98-E99-E100-E101</f>
+        <f>E98-E99-E100-E101-E170</f>
         <v/>
       </c>
       <c r="F102" s="16">
-        <f>F98-F99-F100-F101</f>
+        <f>F98-F99-F100-F101-F170</f>
         <v/>
       </c>
       <c r="G102" s="16">
-        <f>G98-G99-G100-G101</f>
+        <f>G98-G99-G100-G101-G170</f>
         <v/>
       </c>
       <c r="H102" s="16">
-        <f>H98-H99-H100-H101</f>
+        <f>H98-H99-H100-H101-H170</f>
         <v/>
       </c>
       <c r="I102" s="16">
-        <f>I98-I99-I100-I101</f>
+        <f>I98-I99-I100-I101-I170</f>
         <v/>
       </c>
       <c r="J102" s="16">
-        <f>J98-J99-J100-J101</f>
+        <f>J98-J99-J100-J101-J170</f>
         <v/>
       </c>
       <c r="K102" s="16">
-        <f>K98-K99-K100-K101</f>
+        <f>K98-K99-K100-K101-K170</f>
         <v/>
       </c>
       <c r="L102" s="16">
-        <f>L98-L99-L100-L101</f>
+        <f>L98-L99-L100-L101-L170</f>
         <v/>
       </c>
     </row>
@@ -4503,47 +4503,47 @@
         </is>
       </c>
       <c r="B121" s="16">
-        <f>B116-B117-B118-B119-B120</f>
+        <f>B116-B117-B118-B119-B120-B170</f>
         <v/>
       </c>
       <c r="C121" s="16">
-        <f>C116-C117-C118-C119-C120</f>
+        <f>C116-C117-C118-C119-C120-C170</f>
         <v/>
       </c>
       <c r="D121" s="16">
-        <f>D116-D117-D118-D119-D120</f>
+        <f>D116-D117-D118-D119-D120-D170</f>
         <v/>
       </c>
       <c r="E121" s="16">
-        <f>E116-E117-E118-E119-E120</f>
+        <f>E116-E117-E118-E119-E120-E170</f>
         <v/>
       </c>
       <c r="F121" s="16">
-        <f>F116-F117-F118-F119-F120</f>
+        <f>F116-F117-F118-F119-F120-F170</f>
         <v/>
       </c>
       <c r="G121" s="16">
-        <f>G116-G117-G118-G119-G120</f>
+        <f>G116-G117-G118-G119-G120-G170</f>
         <v/>
       </c>
       <c r="H121" s="16">
-        <f>H116-H117-H118-H119-H120</f>
+        <f>H116-H117-H118-H119-H120-H170</f>
         <v/>
       </c>
       <c r="I121" s="16">
-        <f>I116-I117-I118-I119-I120</f>
+        <f>I116-I117-I118-I119-I120-I170</f>
         <v/>
       </c>
       <c r="J121" s="16">
-        <f>J116-J117-J118-J119-J120</f>
+        <f>J116-J117-J118-J119-J120-J170</f>
         <v/>
       </c>
       <c r="K121" s="16">
-        <f>K116-K117-K118-K119-K120</f>
+        <f>K116-K117-K118-K119-K120-K170</f>
         <v/>
       </c>
       <c r="L121" s="16">
-        <f>L116-L117-L118-L119-L120</f>
+        <f>L116-L117-L118-L119-L120-L170</f>
         <v/>
       </c>
     </row>
@@ -5633,7 +5633,7 @@
     <row r="167" ht="30" customHeight="1">
       <c r="A167" s="26" t="inlineStr">
         <is>
-          <t>• Impuestos municipales de Comayagua (industria, comercio y servicios; bienes inmuebles).</t>
+          <t>• Impuesto municipal de Comayagua: Industria, Comercio y Servicios sobre ingresos (Art. 78, escala por millar); el Impuesto sobre Bienes Inmuebles no se cuantifica por ser terreno e instalación propios sin avalúo catastral.</t>
         </is>
       </c>
       <c r="B167" s="27" t="n"/>
@@ -5647,6 +5647,64 @@
       <c r="J167" s="27" t="n"/>
       <c r="K167" s="27" t="n"/>
       <c r="L167" s="28" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>16. IMPUESTO MUNICIPAL DE COMAYAGUA (ICS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>Impuesto de Industria, Comercio y Servicios (sobre ingresos, Art. 78 Ley de Municipalidades)</t>
+        </is>
+      </c>
+      <c r="B170" s="12">
+        <f>0.3/1000*MIN(B42,500000)+0.4/1000*MAX(0,MIN(B42,10000000)-500000)+0.3/1000*MAX(0,MIN(B42,20000000)-10000000)+0.2/1000*MAX(0,MIN(B42,30000000)-20000000)+0.15/1000*MAX(0,B42-30000000)</f>
+        <v/>
+      </c>
+      <c r="C170" s="12">
+        <f>0.3/1000*MIN(C42,500000)+0.4/1000*MAX(0,MIN(C42,10000000)-500000)+0.3/1000*MAX(0,MIN(C42,20000000)-10000000)+0.2/1000*MAX(0,MIN(C42,30000000)-20000000)+0.15/1000*MAX(0,C42-30000000)</f>
+        <v/>
+      </c>
+      <c r="D170" s="12">
+        <f>0.3/1000*MIN(D42,500000)+0.4/1000*MAX(0,MIN(D42,10000000)-500000)+0.3/1000*MAX(0,MIN(D42,20000000)-10000000)+0.2/1000*MAX(0,MIN(D42,30000000)-20000000)+0.15/1000*MAX(0,D42-30000000)</f>
+        <v/>
+      </c>
+      <c r="E170" s="12">
+        <f>0.3/1000*MIN(E42,500000)+0.4/1000*MAX(0,MIN(E42,10000000)-500000)+0.3/1000*MAX(0,MIN(E42,20000000)-10000000)+0.2/1000*MAX(0,MIN(E42,30000000)-20000000)+0.15/1000*MAX(0,E42-30000000)</f>
+        <v/>
+      </c>
+      <c r="F170" s="12">
+        <f>0.3/1000*MIN(F42,500000)+0.4/1000*MAX(0,MIN(F42,10000000)-500000)+0.3/1000*MAX(0,MIN(F42,20000000)-10000000)+0.2/1000*MAX(0,MIN(F42,30000000)-20000000)+0.15/1000*MAX(0,F42-30000000)</f>
+        <v/>
+      </c>
+      <c r="G170" s="12">
+        <f>0.3/1000*MIN(G42,500000)+0.4/1000*MAX(0,MIN(G42,10000000)-500000)+0.3/1000*MAX(0,MIN(G42,20000000)-10000000)+0.2/1000*MAX(0,MIN(G42,30000000)-20000000)+0.15/1000*MAX(0,G42-30000000)</f>
+        <v/>
+      </c>
+      <c r="H170" s="12">
+        <f>0.3/1000*MIN(H42,500000)+0.4/1000*MAX(0,MIN(H42,10000000)-500000)+0.3/1000*MAX(0,MIN(H42,20000000)-10000000)+0.2/1000*MAX(0,MIN(H42,30000000)-20000000)+0.15/1000*MAX(0,H42-30000000)</f>
+        <v/>
+      </c>
+      <c r="I170" s="12">
+        <f>0.3/1000*MIN(I42,500000)+0.4/1000*MAX(0,MIN(I42,10000000)-500000)+0.3/1000*MAX(0,MIN(I42,20000000)-10000000)+0.2/1000*MAX(0,MIN(I42,30000000)-20000000)+0.15/1000*MAX(0,I42-30000000)</f>
+        <v/>
+      </c>
+      <c r="J170" s="12">
+        <f>0.3/1000*MIN(J42,500000)+0.4/1000*MAX(0,MIN(J42,10000000)-500000)+0.3/1000*MAX(0,MIN(J42,20000000)-10000000)+0.2/1000*MAX(0,MIN(J42,30000000)-20000000)+0.15/1000*MAX(0,J42-30000000)</f>
+        <v/>
+      </c>
+      <c r="K170" s="12">
+        <f>0.3/1000*MIN(K42,500000)+0.4/1000*MAX(0,MIN(K42,10000000)-500000)+0.3/1000*MAX(0,MIN(K42,20000000)-10000000)+0.2/1000*MAX(0,MIN(K42,30000000)-20000000)+0.15/1000*MAX(0,K42-30000000)</f>
+        <v/>
+      </c>
+      <c r="L170" s="12">
+        <f>0.3/1000*MIN(L42,500000)+0.4/1000*MAX(0,MIN(L42,10000000)-500000)+0.3/1000*MAX(0,MIN(L42,20000000)-10000000)+0.2/1000*MAX(0,MIN(L42,30000000)-20000000)+0.15/1000*MAX(0,L42-30000000)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="34">
@@ -5859,14 +5917,14 @@
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
         <is>
-          <t>Sin financiamiento: VAN de 15,389,173 Lempiras, TIRM de 40.40%, recuperación en 3.67 años y relación beneficio/costo de 1.23.</t>
+          <t>Sin financiamiento: VAN de 15,370,632 Lempiras, TIRM de 40.38%, recuperación en 3.67 años y relación beneficio/costo de 1.23.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
         <is>
-          <t>Con financiamiento: VAN de 18,282,159 Lempiras, TIRM de 42.49%, recuperación en 3.66 años y relación beneficio/costo de 1.24.</t>
+          <t>Con financiamiento: VAN de 18,261,296 Lempiras, TIRM de 42.46%, recuperación en 3.66 años y relación beneficio/costo de 1.24.</t>
         </is>
       </c>
     </row>
@@ -5890,7 +5948,7 @@
     <row r="31">
       <c r="A31" s="31" t="inlineStr">
         <is>
-          <t>El estudio aplica el impuesto sobre la renta de 25% más 5% de aportación solidaria, la depreciación por línea recta permitida por el reglamento (vehículos entre 10% y 33%, aquí 20%), la seguridad social patronal con su techo de cotización, el aguinaldo y el catorceavo mes del Código del Trabajo, la exención del impuesto sobre ventas para la leche fluida, el arrastre de pérdidas de hasta tres años para la manufactura y los impuestos municipales de Comayagua.</t>
+          <t>El estudio aplica el impuesto sobre la renta de 25% más 5% de aportación solidaria, la depreciación por línea recta permitida por el reglamento (vehículos entre 10% y 33%, aquí 20%), la seguridad social patronal del 7.2% al IHSS más 1% de INFOP con su techo de cotización, el aguinaldo y el catorceavo mes del Código del Trabajo, la exención del impuesto sobre ventas para la leche fluida, el arrastre de pérdidas de hasta tres años para la manufactura, y el impuesto municipal de Comayagua de Industria, Comercio y Servicios sobre los ingresos anuales según la escala de la Ley de Municipalidades.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: corrige nota enganiosa de capital de trabajo (no hay credito de proveedores modelado); ahora describe la realidad: se financia 50% prestamo/50% propios como el resto de la inversion y se recupera en el anio 10
</commit_message>
<xml_diff>
--- a/Estudio_Financiero_Pura.xlsx
+++ b/Estudio_Financiero_Pura.xlsx
@@ -742,7 +742,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Meses de capital de trabajo (crédito de proveedores)</t>
+          <t>Meses de capital de trabajo</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
@@ -5556,7 +5556,7 @@
     <row r="176">
       <c r="A176" s="19" t="inlineStr">
         <is>
-          <t>• Capital de trabajo: 1 mes de costos operativos, financiado con crédito de proveedores.</t>
+          <t>• Capital de trabajo: equivale a 1 mes de costos operativos; forma parte de la inversión inicial (financiada 50% con préstamo y 50% con recursos propios) y se recupera en el año 10.</t>
         </is>
       </c>
     </row>

</xml_diff>